<commit_message>
docs(fp-187): make discounted payback reproducible
</commit_message>
<xml_diff>
--- a/docs/fp-187/flujo-caja-van-tir-fp-187.xlsx
+++ b/docs/fp-187/flujo-caja-van-tir-fp-187.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R59ed84139ef8457f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="2" r:id="R3283e1ac34744342"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flujo mensual" sheetId="3" r:id="R165b826ed7864857"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="4" r:id="R5683e8b88fd5499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="5" r:id="R6a7dcbb556cb4cdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoría" sheetId="6" r:id="R12c1a3570b854dd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rac65bd7fcbe84514"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="2" r:id="R8775895d238b4515"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flujo mensual" sheetId="3" r:id="Rd41631313094426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="4" r:id="R3f59260cd3dd48fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="5" r:id="R5c27532f23d443f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoría" sheetId="6" r:id="R7558cdc4a5e64749"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,14 +18,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="7">
+  <x:numFmts count="8">
     <x:numFmt numFmtId="200" formatCode="$#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="0.00%"/>
-    <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
-    <x:numFmt numFmtId="203" formatCode="#,##0.00"/>
-    <x:numFmt numFmtId="204" formatCode="0.00"/>
-    <x:numFmt numFmtId="205" formatCode="0"/>
-    <x:numFmt numFmtId="206" formatCode="0.0000"/>
+    <x:numFmt numFmtId="202" formatCode="0 &quot;mes&quot;"/>
+    <x:numFmt numFmtId="203" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="204" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="205" formatCode="0.00"/>
+    <x:numFmt numFmtId="206" formatCode="0"/>
+    <x:numFmt numFmtId="207" formatCode="0.0000"/>
   </x:numFmts>
   <x:fonts count="9">
     <x:font>
@@ -116,7 +117,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="45">
+  <x:cellXfs count="46">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -145,6 +146,9 @@
     <x:xf numFmtId="201" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
@@ -165,7 +169,7 @@
     <x:xf numFmtId="201" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="203" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -174,22 +178,22 @@
     <x:xf numFmtId="200" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="203" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="204" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="203" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="204" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="205" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="206" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -216,13 +220,13 @@
     <x:xf numFmtId="201" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="203" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="203" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="204" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -446,84 +450,91 @@
     <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
-      <x:c r="A1" s="43" t="str">
+      <x:c r="A1" s="44" t="str">
         <x:v>FP-187 — Flujo de caja, VAN y TIR de TINV-06</x:v>
       </x:c>
-      <x:c r="B1" s="43"/>
-      <x:c r="C1" s="43"/>
-      <x:c r="D1" s="43"/>
-      <x:c r="E1" s="43"/>
-      <x:c r="F1" s="43"/>
-      <x:c r="G1" s="43"/>
-      <x:c r="H1" s="43"/>
-      <x:c r="I1" s="43"/>
-      <x:c r="J1" s="43"/>
-      <x:c r="K1" s="43"/>
+      <x:c r="B1" s="44"/>
+      <x:c r="C1" s="44"/>
+      <x:c r="D1" s="44"/>
+      <x:c r="E1" s="44"/>
+      <x:c r="F1" s="44"/>
+      <x:c r="G1" s="44"/>
+      <x:c r="H1" s="44"/>
+      <x:c r="I1" s="44"/>
+      <x:c r="J1" s="44"/>
+      <x:c r="K1" s="44"/>
+      <x:c r="L1" s="44"/>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="44" t="str">
+      <x:c r="A2" s="45" t="str">
         <x:v>Modelo financiero vinculado a FP-183/FP-184 con proxies públicos para tasa y costo de mano de obra. Sustituirlos por datos internos cuando estén disponibles.</x:v>
       </x:c>
-      <x:c r="B2" s="44"/>
-      <x:c r="C2" s="44"/>
-      <x:c r="D2" s="44"/>
-      <x:c r="E2" s="44"/>
-      <x:c r="F2" s="44"/>
-      <x:c r="G2" s="44"/>
-      <x:c r="H2" s="44"/>
-      <x:c r="I2" s="44"/>
-      <x:c r="J2" s="44"/>
-      <x:c r="K2" s="44"/>
+      <x:c r="B2" s="45"/>
+      <x:c r="C2" s="45"/>
+      <x:c r="D2" s="45"/>
+      <x:c r="E2" s="45"/>
+      <x:c r="F2" s="45"/>
+      <x:c r="G2" s="45"/>
+      <x:c r="H2" s="45"/>
+      <x:c r="I2" s="45"/>
+      <x:c r="J2" s="45"/>
+      <x:c r="K2" s="45"/>
+      <x:c r="L2" s="45"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="44"/>
-      <x:c r="B3" s="44"/>
-      <x:c r="C3" s="44"/>
-      <x:c r="D3" s="44"/>
-      <x:c r="E3" s="44"/>
-      <x:c r="F3" s="44"/>
-      <x:c r="G3" s="44"/>
-      <x:c r="H3" s="44"/>
-      <x:c r="I3" s="44"/>
-      <x:c r="J3" s="44"/>
-      <x:c r="K3" s="44"/>
+      <x:c r="A3" s="45"/>
+      <x:c r="B3" s="45"/>
+      <x:c r="C3" s="45"/>
+      <x:c r="D3" s="45"/>
+      <x:c r="E3" s="45"/>
+      <x:c r="F3" s="45"/>
+      <x:c r="G3" s="45"/>
+      <x:c r="H3" s="45"/>
+      <x:c r="I3" s="45"/>
+      <x:c r="J3" s="45"/>
+      <x:c r="K3" s="45"/>
+      <x:c r="L3" s="45"/>
     </x:row>
     <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A4" s="36" t="str">
+      <x:c r="A4" s="37" t="str">
         <x:v>Indicador</x:v>
       </x:c>
-      <x:c r="B4" s="36" t="str">
+      <x:c r="B4" s="37" t="str">
         <x:v>Región</x:v>
       </x:c>
-      <x:c r="C4" s="36" t="str">
+      <x:c r="C4" s="37" t="str">
         <x:v>TCO base cloud 60m</x:v>
       </x:c>
-      <x:c r="D4" s="36" t="str">
+      <x:c r="D4" s="37" t="str">
         <x:v>TCO optimizado cloud 60m</x:v>
       </x:c>
-      <x:c r="E4" s="36" t="str">
+      <x:c r="E4" s="37" t="str">
         <x:v>Ahorro bruto 60m</x:v>
       </x:c>
-      <x:c r="F4" s="36" t="str">
+      <x:c r="F4" s="37" t="str">
         <x:v>Operación 60m</x:v>
       </x:c>
-      <x:c r="G4" s="36" t="str">
+      <x:c r="G4" s="37" t="str">
         <x:v>Implementación inicial</x:v>
       </x:c>
-      <x:c r="H4" s="36" t="str">
+      <x:c r="H4" s="37" t="str">
         <x:v>VAN bruto ahorro</x:v>
       </x:c>
-      <x:c r="I4" s="36" t="str">
+      <x:c r="I4" s="37" t="str">
         <x:v>VAN incremental</x:v>
       </x:c>
-      <x:c r="J4" s="36" t="str">
+      <x:c r="J4" s="37" t="str">
         <x:v>TIR incremental anual</x:v>
       </x:c>
-      <x:c r="K4" s="36" t="str">
+      <x:c r="K4" s="37" t="str">
+        <x:v>PRI descontado</x:v>
+      </x:c>
+      <x:c r="L4" s="37" t="str">
         <x:v>Estado</x:v>
       </x:c>
     </x:row>
@@ -566,7 +577,11 @@
         <x:f>IF(OR(G5="",G5&lt;=0),"",(1+IRR('Flujo mensual'!I7:I67))^12-1)</x:f>
         <x:v>0.4391345109616156</x:v>
       </x:c>
-      <x:c r="K5" s="14" t="str">
+      <x:c r="K5" s="14" t="n">
+        <x:f>IF(COUNT('Flujo mensual'!Z7:Z67)=0,"No recupera en 60 meses",SUM('Flujo mensual'!Z7:Z67))</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="L5" s="15" t="str">
         <x:f>IF(OR(G5="",Supuestos!$B$13="",Supuestos!$B$14=""),"Provisional: completar inputs",Supuestos!$B$18)</x:f>
         <x:v>Provisional: proxies públicos</x:v>
       </x:c>
@@ -611,86 +626,95 @@
         <x:v>-0.002138745694702626</x:v>
       </x:c>
       <x:c r="K6" s="14" t="str">
+        <x:f>IF(COUNT('Flujo mensual'!AA7:AA67)=0,"No recupera en 60 meses",SUM('Flujo mensual'!AA7:AA67))</x:f>
+        <x:v>No recupera en 60 meses</x:v>
+      </x:c>
+      <x:c r="L6" s="15" t="str">
         <x:f>IF(OR(G6="",Supuestos!$B$13="",Supuestos!$B$14=""),"Provisional: completar inputs",Supuestos!$B$18)</x:f>
         <x:v>Provisional: proxies públicos</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="44"/>
-      <x:c r="B7" s="44"/>
-      <x:c r="C7" s="44"/>
-      <x:c r="D7" s="44"/>
-      <x:c r="E7" s="44"/>
-      <x:c r="F7" s="44"/>
-      <x:c r="G7" s="44"/>
-      <x:c r="H7" s="44"/>
-      <x:c r="I7" s="44"/>
-      <x:c r="J7" s="44"/>
-      <x:c r="K7" s="44"/>
+      <x:c r="A7" s="45"/>
+      <x:c r="B7" s="45"/>
+      <x:c r="C7" s="45"/>
+      <x:c r="D7" s="45"/>
+      <x:c r="E7" s="45"/>
+      <x:c r="F7" s="45"/>
+      <x:c r="G7" s="45"/>
+      <x:c r="H7" s="45"/>
+      <x:c r="I7" s="45"/>
+      <x:c r="J7" s="45"/>
+      <x:c r="K7" s="45"/>
+      <x:c r="L7" s="45"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="44"/>
-      <x:c r="B8" s="44"/>
-      <x:c r="C8" s="44"/>
-      <x:c r="D8" s="44"/>
-      <x:c r="E8" s="44"/>
-      <x:c r="F8" s="44"/>
-      <x:c r="G8" s="44"/>
-      <x:c r="H8" s="44"/>
-      <x:c r="I8" s="44"/>
-      <x:c r="J8" s="44"/>
-      <x:c r="K8" s="44"/>
+      <x:c r="A8" s="45"/>
+      <x:c r="B8" s="45"/>
+      <x:c r="C8" s="45"/>
+      <x:c r="D8" s="45"/>
+      <x:c r="E8" s="45"/>
+      <x:c r="F8" s="45"/>
+      <x:c r="G8" s="45"/>
+      <x:c r="H8" s="45"/>
+      <x:c r="I8" s="45"/>
+      <x:c r="J8" s="45"/>
+      <x:c r="K8" s="45"/>
+      <x:c r="L8" s="45"/>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="37" t="str">
-        <x:v>Lectura: VAN bruto representa el ahorro cloud descontado. VAN incremental descuenta implementación y operación FinOps mensual. TIR es anualizada desde el flujo incremental neto.</x:v>
-      </x:c>
-      <x:c r="B9" s="37"/>
-      <x:c r="C9" s="37"/>
-      <x:c r="D9" s="37"/>
-      <x:c r="E9" s="37"/>
-      <x:c r="F9" s="37"/>
-      <x:c r="G9" s="37"/>
-      <x:c r="H9" s="37"/>
-      <x:c r="I9" s="37"/>
-      <x:c r="J9" s="37"/>
-      <x:c r="K9" s="37"/>
+      <x:c r="A9" s="38" t="str">
+        <x:v>Lectura: VAN bruto representa el ahorro cloud descontado. VAN incremental descuenta implementación y operación FinOps mensual. TIR se anualiza desde el flujo incremental neto. PRI es el primer mes cuyo flujo descontado acumulado es no negativo.</x:v>
+      </x:c>
+      <x:c r="B9" s="38"/>
+      <x:c r="C9" s="38"/>
+      <x:c r="D9" s="38"/>
+      <x:c r="E9" s="38"/>
+      <x:c r="F9" s="38"/>
+      <x:c r="G9" s="38"/>
+      <x:c r="H9" s="38"/>
+      <x:c r="I9" s="38"/>
+      <x:c r="J9" s="38"/>
+      <x:c r="K9" s="38"/>
+      <x:c r="L9" s="38"/>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="37"/>
-      <x:c r="B10" s="37"/>
-      <x:c r="C10" s="37"/>
-      <x:c r="D10" s="37"/>
-      <x:c r="E10" s="37"/>
-      <x:c r="F10" s="37"/>
-      <x:c r="G10" s="37"/>
-      <x:c r="H10" s="37"/>
-      <x:c r="I10" s="37"/>
-      <x:c r="J10" s="37"/>
-      <x:c r="K10" s="37"/>
+      <x:c r="A10" s="38"/>
+      <x:c r="B10" s="38"/>
+      <x:c r="C10" s="38"/>
+      <x:c r="D10" s="38"/>
+      <x:c r="E10" s="38"/>
+      <x:c r="F10" s="38"/>
+      <x:c r="G10" s="38"/>
+      <x:c r="H10" s="38"/>
+      <x:c r="I10" s="38"/>
+      <x:c r="J10" s="38"/>
+      <x:c r="K10" s="38"/>
+      <x:c r="L10" s="38"/>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="37" t="str">
+      <x:c r="A11" s="38" t="str">
         <x:v>Limitación: tasa, tarifa y esfuerzo usan proxies públicos/estimaciones de ingeniería, no datos internos. El escenario es defendible como estimación provisional, no como presupuesto contractual.</x:v>
       </x:c>
-      <x:c r="B11" s="37"/>
-      <x:c r="C11" s="37"/>
-      <x:c r="D11" s="37"/>
-      <x:c r="E11" s="37"/>
-      <x:c r="F11" s="37"/>
-      <x:c r="G11" s="37"/>
-      <x:c r="H11" s="37"/>
-      <x:c r="I11" s="37"/>
-      <x:c r="J11" s="37"/>
-      <x:c r="K11" s="37"/>
+      <x:c r="B11" s="38"/>
+      <x:c r="C11" s="38"/>
+      <x:c r="D11" s="38"/>
+      <x:c r="E11" s="38"/>
+      <x:c r="F11" s="38"/>
+      <x:c r="G11" s="38"/>
+      <x:c r="H11" s="38"/>
+      <x:c r="I11" s="38"/>
+      <x:c r="J11" s="38"/>
+      <x:c r="K11" s="38"/>
+      <x:c r="L11" s="38"/>
     </x:row>
     <x:row r="12"/>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:K1"/>
-    <x:mergeCell ref="A2:K2"/>
-    <x:mergeCell ref="A9:K9"/>
-    <x:mergeCell ref="A11:K11"/>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
+    <x:mergeCell ref="A9:L9"/>
+    <x:mergeCell ref="A11:L11"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -707,50 +731,50 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="43" t="str">
+      <x:c r="A1" s="44" t="str">
         <x:v>FP-187 — Supuestos financieros y parámetros editables</x:v>
       </x:c>
-      <x:c r="B1" s="43"/>
-      <x:c r="C1" s="43"/>
-      <x:c r="D1" s="43"/>
+      <x:c r="B1" s="44"/>
+      <x:c r="C1" s="44"/>
+      <x:c r="D1" s="44"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="44"/>
-      <x:c r="B2" s="44"/>
-      <x:c r="C2" s="44"/>
-      <x:c r="D2" s="44"/>
+      <x:c r="A2" s="45"/>
+      <x:c r="B2" s="45"/>
+      <x:c r="C2" s="45"/>
+      <x:c r="D2" s="45"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="44" t="str">
+      <x:c r="A3" s="45" t="str">
         <x:v>Las celdas amarillas contienen proxies públicos o estimaciones editables. Los valores no representan tarifas internas ni una cotización contractual.</x:v>
       </x:c>
-      <x:c r="B3" s="44"/>
-      <x:c r="C3" s="44"/>
-      <x:c r="D3" s="44"/>
+      <x:c r="B3" s="45"/>
+      <x:c r="C3" s="45"/>
+      <x:c r="D3" s="45"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="44"/>
-      <x:c r="B4" s="44"/>
-      <x:c r="C4" s="44"/>
-      <x:c r="D4" s="44"/>
+      <x:c r="A4" s="45"/>
+      <x:c r="B4" s="45"/>
+      <x:c r="C4" s="45"/>
+      <x:c r="D4" s="45"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="44"/>
-      <x:c r="B5" s="44"/>
-      <x:c r="C5" s="44"/>
-      <x:c r="D5" s="44"/>
+      <x:c r="A5" s="45"/>
+      <x:c r="B5" s="45"/>
+      <x:c r="C5" s="45"/>
+      <x:c r="D5" s="45"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="36" t="str">
+      <x:c r="A6" s="37" t="str">
         <x:v>Variable</x:v>
       </x:c>
-      <x:c r="B6" s="36" t="str">
+      <x:c r="B6" s="37" t="str">
         <x:v>Valor</x:v>
       </x:c>
-      <x:c r="C6" s="36" t="str">
+      <x:c r="C6" s="37" t="str">
         <x:v>Unidad</x:v>
       </x:c>
-      <x:c r="D6" s="36" t="str">
+      <x:c r="D6" s="37" t="str">
         <x:v>Origen / regla</x:v>
       </x:c>
     </x:row>
@@ -758,7 +782,7 @@
       <x:c r="A7" s="11" t="str">
         <x:v>Horizonte</x:v>
       </x:c>
-      <x:c r="B7" s="14" t="n">
+      <x:c r="B7" s="15" t="n">
         <x:v>60</x:v>
       </x:c>
       <x:c r="C7" s="11" t="str">
@@ -772,7 +796,7 @@
       <x:c r="A8" s="11" t="str">
         <x:v>Tasa descuento anual</x:v>
       </x:c>
-      <x:c r="B8" s="38" t="n">
+      <x:c r="B8" s="39" t="n">
         <x:v>0.055</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
@@ -786,7 +810,7 @@
       <x:c r="A9" s="11" t="str">
         <x:v>Tasa descuento mensual</x:v>
       </x:c>
-      <x:c r="B9" s="38" t="n">
+      <x:c r="B9" s="39" t="n">
         <x:f>(1+B8)^(1/12)-1</x:f>
         <x:v>0.004471698917043021</x:v>
       </x:c>
@@ -801,7 +825,7 @@
       <x:c r="A10" s="11" t="str">
         <x:v>Fecha inicio</x:v>
       </x:c>
-      <x:c r="B10" s="39" t="n">
+      <x:c r="B10" s="40" t="n">
         <x:v>46023</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
@@ -815,7 +839,7 @@
       <x:c r="A11" s="11" t="str">
         <x:v>Inversión inicial Chile</x:v>
       </x:c>
-      <x:c r="B11" s="40" t="n">
+      <x:c r="B11" s="41" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C11" s="11" t="str">
@@ -829,7 +853,7 @@
       <x:c r="A12" s="11" t="str">
         <x:v>Inversión inicial East US</x:v>
       </x:c>
-      <x:c r="B12" s="40" t="n">
+      <x:c r="B12" s="41" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
@@ -843,7 +867,7 @@
       <x:c r="A13" s="11" t="str">
         <x:v>Horas operación FinOps mensuales</x:v>
       </x:c>
-      <x:c r="B13" s="14" t="n">
+      <x:c r="B13" s="15" t="n">
         <x:f>B30</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -858,7 +882,7 @@
       <x:c r="A14" s="11" t="str">
         <x:v>Tarifa operación</x:v>
       </x:c>
-      <x:c r="B14" s="14" t="n">
+      <x:c r="B14" s="15" t="n">
         <x:f>B28</x:f>
         <x:v>8.53452616399676</x:v>
       </x:c>
@@ -873,7 +897,7 @@
       <x:c r="A15" s="11" t="str">
         <x:v>Implementación optimización Chile</x:v>
       </x:c>
-      <x:c r="B15" s="40" t="n">
+      <x:c r="B15" s="41" t="n">
         <x:f>B29*B14</x:f>
         <x:v>426.72630819983806</x:v>
       </x:c>
@@ -888,7 +912,7 @@
       <x:c r="A16" s="11" t="str">
         <x:v>Implementación optimización East US</x:v>
       </x:c>
-      <x:c r="B16" s="40" t="n">
+      <x:c r="B16" s="41" t="n">
         <x:f>B29*B14</x:f>
         <x:v>426.72630819983806</x:v>
       </x:c>
@@ -903,7 +927,7 @@
       <x:c r="A17" s="11" t="str">
         <x:v>Moneda</x:v>
       </x:c>
-      <x:c r="B17" s="14" t="str">
+      <x:c r="B17" s="15" t="str">
         <x:v>USD</x:v>
       </x:c>
       <x:c r="C17" s="11" t="str">
@@ -917,7 +941,7 @@
       <x:c r="A18" s="11" t="str">
         <x:v>Estado aprobación</x:v>
       </x:c>
-      <x:c r="B18" s="14" t="str">
+      <x:c r="B18" s="15" t="str">
         <x:v>Provisional: proxies públicos</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
@@ -931,7 +955,7 @@
       <x:c r="A19" s="11" t="str">
         <x:v>Ahorro bruto FP-184 Chile</x:v>
       </x:c>
-      <x:c r="B19" s="40" t="n">
+      <x:c r="B19" s="41" t="n">
         <x:v>1453.152</x:v>
       </x:c>
       <x:c r="C19" s="11" t="str">
@@ -945,7 +969,7 @@
       <x:c r="A20" s="11" t="str">
         <x:v>Ahorro bruto FP-184 East US</x:v>
       </x:c>
-      <x:c r="B20" s="40" t="n">
+      <x:c r="B20" s="41" t="n">
         <x:v>936.48</x:v>
       </x:c>
       <x:c r="C20" s="11" t="str">
@@ -959,7 +983,7 @@
       <x:c r="A21" s="11" t="str">
         <x:v>Ahorro mensual Chile</x:v>
       </x:c>
-      <x:c r="B21" s="40" t="n">
+      <x:c r="B21" s="41" t="n">
         <x:f>B19/B7</x:f>
         <x:v>24.2192</x:v>
       </x:c>
@@ -974,7 +998,7 @@
       <x:c r="A22" s="11" t="str">
         <x:v>Ahorro mensual East US</x:v>
       </x:c>
-      <x:c r="B22" s="40" t="n">
+      <x:c r="B22" s="41" t="n">
         <x:f>B20/B7</x:f>
         <x:v>15.608</x:v>
       </x:c>
@@ -989,7 +1013,7 @@
       <x:c r="A23" s="11" t="str">
         <x:v>Nota de modelación</x:v>
       </x:c>
-      <x:c r="B23" s="14" t="str">
+      <x:c r="B23" s="15" t="str">
         <x:v>El flujo incremental mide la decisión de optimización; no sustituye al TCO.</x:v>
       </x:c>
       <x:c r="C23" s="11" t="str">
@@ -1003,7 +1027,7 @@
       <x:c r="A24" s="11" t="str">
         <x:v>Tipo de cambio</x:v>
       </x:c>
-      <x:c r="B24" s="41" t="n">
+      <x:c r="B24" s="42" t="n">
         <x:v>954.85</x:v>
       </x:c>
       <x:c r="C24" s="11" t="str">
@@ -1017,7 +1041,7 @@
       <x:c r="A25" s="11" t="str">
         <x:v>Ingreso neto mensual universitario</x:v>
       </x:c>
-      <x:c r="B25" s="41" t="n">
+      <x:c r="B25" s="42" t="n">
         <x:v>1483153</x:v>
       </x:c>
       <x:c r="C25" s="11" t="str">
@@ -1031,7 +1055,7 @@
       <x:c r="A26" s="11" t="str">
         <x:v>Jornada semanal</x:v>
       </x:c>
-      <x:c r="B26" s="14" t="n">
+      <x:c r="B26" s="15" t="n">
         <x:v>42</x:v>
       </x:c>
       <x:c r="C26" s="11" t="str">
@@ -1045,7 +1069,7 @@
       <x:c r="A27" s="11" t="str">
         <x:v>Horas laborales mensuales</x:v>
       </x:c>
-      <x:c r="B27" s="41" t="n">
+      <x:c r="B27" s="42" t="n">
         <x:f>B26*52/12</x:f>
         <x:v>182</x:v>
       </x:c>
@@ -1060,7 +1084,7 @@
       <x:c r="A28" s="11" t="str">
         <x:v>Tarifa horaria proxy</x:v>
       </x:c>
-      <x:c r="B28" s="41" t="n">
+      <x:c r="B28" s="42" t="n">
         <x:f>B25/B27/B24</x:f>
         <x:v>8.53452616399676</x:v>
       </x:c>
@@ -1075,7 +1099,7 @@
       <x:c r="A29" s="11" t="str">
         <x:v>Horas implementación por escenario</x:v>
       </x:c>
-      <x:c r="B29" s="41" t="n">
+      <x:c r="B29" s="42" t="n">
         <x:f>B40</x:f>
         <x:v>50</x:v>
       </x:c>
@@ -1090,7 +1114,7 @@
       <x:c r="A30" s="11" t="str">
         <x:v>Horas operación por escenario</x:v>
       </x:c>
-      <x:c r="B30" s="41" t="n">
+      <x:c r="B30" s="42" t="n">
         <x:f>B47</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -1105,7 +1129,7 @@
       <x:c r="A31" s="11" t="str">
         <x:v>Alcance financiero</x:v>
       </x:c>
-      <x:c r="B31" s="14" t="str">
+      <x:c r="B31" s="15" t="str">
         <x:v>USD constantes; sin impuestos, inflación ni valor residual</x:v>
       </x:c>
       <x:c r="C31" s="11" t="str">
@@ -1116,174 +1140,174 @@
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="44"/>
-      <x:c r="B32" s="44"/>
-      <x:c r="C32" s="44"/>
-      <x:c r="D32" s="44"/>
+      <x:c r="A32" s="45"/>
+      <x:c r="B32" s="45"/>
+      <x:c r="C32" s="45"/>
+      <x:c r="D32" s="45"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="44"/>
-      <x:c r="B33" s="44"/>
-      <x:c r="C33" s="44"/>
-      <x:c r="D33" s="44"/>
+      <x:c r="A33" s="45"/>
+      <x:c r="B33" s="45"/>
+      <x:c r="C33" s="45"/>
+      <x:c r="D33" s="45"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="36" t="str">
+      <x:c r="A34" s="37" t="str">
         <x:v>Implementación por escenario</x:v>
       </x:c>
-      <x:c r="B34" s="36" t="str">
+      <x:c r="B34" s="37" t="str">
         <x:v>Horas</x:v>
       </x:c>
-      <x:c r="C34" s="36" t="str">
+      <x:c r="C34" s="37" t="str">
         <x:v>Base de estimación</x:v>
       </x:c>
-      <x:c r="D34" s="44"/>
+      <x:c r="D34" s="45"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="11" t="str">
         <x:v>Revisión de línea base y plan</x:v>
       </x:c>
-      <x:c r="B35" s="27" t="n">
+      <x:c r="B35" s="28" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C35" s="11" t="str">
         <x:v>Conciliar FP-183/FP-184 y preparar cambio</x:v>
       </x:c>
-      <x:c r="D35" s="44"/>
+      <x:c r="D35" s="45"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="11" t="str">
         <x:v>Rightsizing PostgreSQL</x:v>
       </x:c>
-      <x:c r="B36" s="27" t="n">
+      <x:c r="B36" s="28" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="C36" s="11" t="str">
         <x:v>Analizar, configurar y probar</x:v>
       </x:c>
-      <x:c r="D36" s="44"/>
+      <x:c r="D36" s="45"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="11" t="str">
         <x:v>Programación de no producción</x:v>
       </x:c>
-      <x:c r="B37" s="27" t="n">
+      <x:c r="B37" s="28" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="C37" s="11" t="str">
         <x:v>Automatización, prueba y rollback</x:v>
       </x:c>
-      <x:c r="D37" s="44"/>
+      <x:c r="D37" s="45"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="11" t="str">
         <x:v>Retención e ingesta de logs</x:v>
       </x:c>
-      <x:c r="B38" s="27" t="n">
+      <x:c r="B38" s="28" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C38" s="11" t="str">
         <x:v>Política, configuración y validación</x:v>
       </x:c>
-      <x:c r="D38" s="44"/>
+      <x:c r="D38" s="45"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="11" t="str">
         <x:v>Control, documentación y cierre</x:v>
       </x:c>
-      <x:c r="B39" s="27" t="n">
+      <x:c r="B39" s="28" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="C39" s="11" t="str">
         <x:v>Evidencia, revisión y seguimiento</x:v>
       </x:c>
-      <x:c r="D39" s="44"/>
+      <x:c r="D39" s="45"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="11" t="str">
         <x:v>Total</x:v>
       </x:c>
-      <x:c r="B40" s="27" t="n">
+      <x:c r="B40" s="28" t="n">
         <x:f>SUM(B35:B39)</x:f>
         <x:v>50</x:v>
       </x:c>
       <x:c r="C40" s="11" t="str">
         <x:v>Suma del esfuerzo por alternativa regional</x:v>
       </x:c>
-      <x:c r="D40" s="44"/>
+      <x:c r="D40" s="45"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="44"/>
-      <x:c r="B41" s="44"/>
-      <x:c r="C41" s="44"/>
-      <x:c r="D41" s="44"/>
+      <x:c r="A41" s="45"/>
+      <x:c r="B41" s="45"/>
+      <x:c r="C41" s="45"/>
+      <x:c r="D41" s="45"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="44"/>
-      <x:c r="B42" s="44"/>
-      <x:c r="C42" s="44"/>
-      <x:c r="D42" s="44"/>
+      <x:c r="A42" s="45"/>
+      <x:c r="B42" s="45"/>
+      <x:c r="C42" s="45"/>
+      <x:c r="D42" s="45"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="36" t="str">
+      <x:c r="A43" s="37" t="str">
         <x:v>Operación FinOps mensual</x:v>
       </x:c>
-      <x:c r="B43" s="36" t="str">
+      <x:c r="B43" s="37" t="str">
         <x:v>Horas/mes</x:v>
       </x:c>
-      <x:c r="C43" s="36" t="str">
+      <x:c r="C43" s="37" t="str">
         <x:v>Base de estimación</x:v>
       </x:c>
-      <x:c r="D43" s="44"/>
+      <x:c r="D43" s="45"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="11" t="str">
         <x:v>Revisión de costo y uso</x:v>
       </x:c>
-      <x:c r="B44" s="27" t="n">
+      <x:c r="B44" s="28" t="n">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="C44" s="11" t="str">
         <x:v>Revisión mensual de una carga pequeña</x:v>
       </x:c>
-      <x:c r="D44" s="44"/>
+      <x:c r="D44" s="45"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="11" t="str">
         <x:v>Anomalías, presupuesto y reporte</x:v>
       </x:c>
-      <x:c r="B45" s="27" t="n">
+      <x:c r="B45" s="28" t="n">
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="C45" s="11" t="str">
         <x:v>Control mensual</x:v>
       </x:c>
-      <x:c r="D45" s="44"/>
+      <x:c r="D45" s="45"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="11" t="str">
         <x:v>Seguimiento de optimización</x:v>
       </x:c>
-      <x:c r="B46" s="27" t="n">
+      <x:c r="B46" s="28" t="n">
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="C46" s="11" t="str">
         <x:v>Revisión de acciones abiertas</x:v>
       </x:c>
-      <x:c r="D46" s="44"/>
+      <x:c r="D46" s="45"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="11" t="str">
         <x:v>Total</x:v>
       </x:c>
-      <x:c r="B47" s="27" t="n">
+      <x:c r="B47" s="28" t="n">
         <x:f>SUM(B44:B46)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C47" s="11" t="str">
         <x:v>Suma mensual por alternativa regional</x:v>
       </x:c>
-      <x:c r="D47" s="44"/>
+      <x:c r="D47" s="45"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1321,213 +1345,249 @@
     <x:col min="21" max="21" width="17" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="19" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="19" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="20" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="20" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="18" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="43" t="str">
+      <x:c r="A1" s="44" t="str">
         <x:v>FP-187 — Flujo mensual base, optimizado e incremental</x:v>
       </x:c>
-      <x:c r="B1" s="43"/>
-      <x:c r="C1" s="43"/>
-      <x:c r="D1" s="43"/>
-      <x:c r="E1" s="43"/>
-      <x:c r="F1" s="43"/>
-      <x:c r="G1" s="43"/>
-      <x:c r="H1" s="43"/>
-      <x:c r="I1" s="43"/>
-      <x:c r="J1" s="43"/>
-      <x:c r="K1" s="43"/>
-      <x:c r="L1" s="43"/>
-      <x:c r="M1" s="43"/>
-      <x:c r="N1" s="43"/>
-      <x:c r="O1" s="43"/>
-      <x:c r="P1" s="43"/>
-      <x:c r="Q1" s="43"/>
-      <x:c r="R1" s="43"/>
-      <x:c r="S1" s="43"/>
-      <x:c r="T1" s="43"/>
-      <x:c r="U1" s="43"/>
-      <x:c r="V1" s="43"/>
-      <x:c r="W1" s="43"/>
+      <x:c r="B1" s="44"/>
+      <x:c r="C1" s="44"/>
+      <x:c r="D1" s="44"/>
+      <x:c r="E1" s="44"/>
+      <x:c r="F1" s="44"/>
+      <x:c r="G1" s="44"/>
+      <x:c r="H1" s="44"/>
+      <x:c r="I1" s="44"/>
+      <x:c r="J1" s="44"/>
+      <x:c r="K1" s="44"/>
+      <x:c r="L1" s="44"/>
+      <x:c r="M1" s="44"/>
+      <x:c r="N1" s="44"/>
+      <x:c r="O1" s="44"/>
+      <x:c r="P1" s="44"/>
+      <x:c r="Q1" s="44"/>
+      <x:c r="R1" s="44"/>
+      <x:c r="S1" s="44"/>
+      <x:c r="T1" s="44"/>
+      <x:c r="U1" s="44"/>
+      <x:c r="V1" s="44"/>
+      <x:c r="W1" s="44"/>
+      <x:c r="X1" s="44"/>
+      <x:c r="Y1" s="44"/>
+      <x:c r="Z1" s="44"/>
+      <x:c r="AA1" s="44"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="44"/>
-      <x:c r="B2" s="44"/>
-      <x:c r="C2" s="44"/>
-      <x:c r="D2" s="44"/>
-      <x:c r="E2" s="44"/>
-      <x:c r="F2" s="44"/>
-      <x:c r="G2" s="44"/>
-      <x:c r="H2" s="44"/>
-      <x:c r="I2" s="44"/>
-      <x:c r="J2" s="44"/>
-      <x:c r="K2" s="44"/>
-      <x:c r="L2" s="44"/>
-      <x:c r="M2" s="44"/>
-      <x:c r="N2" s="44"/>
-      <x:c r="O2" s="44"/>
-      <x:c r="P2" s="44"/>
-      <x:c r="Q2" s="44"/>
-      <x:c r="R2" s="44"/>
-      <x:c r="S2" s="44"/>
-      <x:c r="T2" s="44"/>
-      <x:c r="U2" s="44"/>
-      <x:c r="V2" s="44"/>
-      <x:c r="W2" s="44"/>
+      <x:c r="A2" s="45"/>
+      <x:c r="B2" s="45"/>
+      <x:c r="C2" s="45"/>
+      <x:c r="D2" s="45"/>
+      <x:c r="E2" s="45"/>
+      <x:c r="F2" s="45"/>
+      <x:c r="G2" s="45"/>
+      <x:c r="H2" s="45"/>
+      <x:c r="I2" s="45"/>
+      <x:c r="J2" s="45"/>
+      <x:c r="K2" s="45"/>
+      <x:c r="L2" s="45"/>
+      <x:c r="M2" s="45"/>
+      <x:c r="N2" s="45"/>
+      <x:c r="O2" s="45"/>
+      <x:c r="P2" s="45"/>
+      <x:c r="Q2" s="45"/>
+      <x:c r="R2" s="45"/>
+      <x:c r="S2" s="45"/>
+      <x:c r="T2" s="45"/>
+      <x:c r="U2" s="45"/>
+      <x:c r="V2" s="45"/>
+      <x:c r="W2" s="45"/>
+      <x:c r="X2" s="45"/>
+      <x:c r="Y2" s="45"/>
+      <x:c r="Z2" s="45"/>
+      <x:c r="AA2" s="45"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="44" t="str">
-        <x:v>Mes 0 contiene las inversiones iniciales. Meses 1–60 enlazan costos cloud de FP-183 y ahorro bruto de FP-184. El flujo incremental es el usado para VAN/TIR.</x:v>
-      </x:c>
-      <x:c r="B3" s="44"/>
-      <x:c r="C3" s="44"/>
-      <x:c r="D3" s="44"/>
-      <x:c r="E3" s="44"/>
-      <x:c r="F3" s="44"/>
-      <x:c r="G3" s="44"/>
-      <x:c r="H3" s="44"/>
-      <x:c r="I3" s="44"/>
-      <x:c r="J3" s="44"/>
-      <x:c r="K3" s="44"/>
-      <x:c r="L3" s="44"/>
-      <x:c r="M3" s="44"/>
-      <x:c r="N3" s="44"/>
-      <x:c r="O3" s="44"/>
-      <x:c r="P3" s="44"/>
-      <x:c r="Q3" s="44"/>
-      <x:c r="R3" s="44"/>
-      <x:c r="S3" s="44"/>
-      <x:c r="T3" s="44"/>
-      <x:c r="U3" s="44"/>
-      <x:c r="V3" s="44"/>
-      <x:c r="W3" s="44"/>
+      <x:c r="A3" s="45" t="str">
+        <x:v>Mes 0 contiene las inversiones iniciales. Meses 1–60 enlazan costos cloud de FP-183 y ahorro bruto de FP-184. El flujo incremental descontado y su acumulado determinan VAN, TIR y PRI.</x:v>
+      </x:c>
+      <x:c r="B3" s="45"/>
+      <x:c r="C3" s="45"/>
+      <x:c r="D3" s="45"/>
+      <x:c r="E3" s="45"/>
+      <x:c r="F3" s="45"/>
+      <x:c r="G3" s="45"/>
+      <x:c r="H3" s="45"/>
+      <x:c r="I3" s="45"/>
+      <x:c r="J3" s="45"/>
+      <x:c r="K3" s="45"/>
+      <x:c r="L3" s="45"/>
+      <x:c r="M3" s="45"/>
+      <x:c r="N3" s="45"/>
+      <x:c r="O3" s="45"/>
+      <x:c r="P3" s="45"/>
+      <x:c r="Q3" s="45"/>
+      <x:c r="R3" s="45"/>
+      <x:c r="S3" s="45"/>
+      <x:c r="T3" s="45"/>
+      <x:c r="U3" s="45"/>
+      <x:c r="V3" s="45"/>
+      <x:c r="W3" s="45"/>
+      <x:c r="X3" s="45"/>
+      <x:c r="Y3" s="45"/>
+      <x:c r="Z3" s="45"/>
+      <x:c r="AA3" s="45"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="44"/>
-      <x:c r="B4" s="44"/>
-      <x:c r="C4" s="44"/>
-      <x:c r="D4" s="44"/>
-      <x:c r="E4" s="44"/>
-      <x:c r="F4" s="44"/>
-      <x:c r="G4" s="44"/>
-      <x:c r="H4" s="44"/>
-      <x:c r="I4" s="44"/>
-      <x:c r="J4" s="44"/>
-      <x:c r="K4" s="44"/>
-      <x:c r="L4" s="44"/>
-      <x:c r="M4" s="44"/>
-      <x:c r="N4" s="44"/>
-      <x:c r="O4" s="44"/>
-      <x:c r="P4" s="44"/>
-      <x:c r="Q4" s="44"/>
-      <x:c r="R4" s="44"/>
-      <x:c r="S4" s="44"/>
-      <x:c r="T4" s="44"/>
-      <x:c r="U4" s="44"/>
-      <x:c r="V4" s="44"/>
-      <x:c r="W4" s="44"/>
+      <x:c r="A4" s="45"/>
+      <x:c r="B4" s="45"/>
+      <x:c r="C4" s="45"/>
+      <x:c r="D4" s="45"/>
+      <x:c r="E4" s="45"/>
+      <x:c r="F4" s="45"/>
+      <x:c r="G4" s="45"/>
+      <x:c r="H4" s="45"/>
+      <x:c r="I4" s="45"/>
+      <x:c r="J4" s="45"/>
+      <x:c r="K4" s="45"/>
+      <x:c r="L4" s="45"/>
+      <x:c r="M4" s="45"/>
+      <x:c r="N4" s="45"/>
+      <x:c r="O4" s="45"/>
+      <x:c r="P4" s="45"/>
+      <x:c r="Q4" s="45"/>
+      <x:c r="R4" s="45"/>
+      <x:c r="S4" s="45"/>
+      <x:c r="T4" s="45"/>
+      <x:c r="U4" s="45"/>
+      <x:c r="V4" s="45"/>
+      <x:c r="W4" s="45"/>
+      <x:c r="X4" s="45"/>
+      <x:c r="Y4" s="45"/>
+      <x:c r="Z4" s="45"/>
+      <x:c r="AA4" s="45"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="44"/>
-      <x:c r="B5" s="44"/>
-      <x:c r="C5" s="44"/>
-      <x:c r="D5" s="44"/>
-      <x:c r="E5" s="44"/>
-      <x:c r="F5" s="44"/>
-      <x:c r="G5" s="44"/>
-      <x:c r="H5" s="44"/>
-      <x:c r="I5" s="44"/>
-      <x:c r="J5" s="44"/>
-      <x:c r="K5" s="44"/>
-      <x:c r="L5" s="44"/>
-      <x:c r="M5" s="44"/>
-      <x:c r="N5" s="44"/>
-      <x:c r="O5" s="44"/>
-      <x:c r="P5" s="44"/>
-      <x:c r="Q5" s="44"/>
-      <x:c r="R5" s="44"/>
-      <x:c r="S5" s="44"/>
-      <x:c r="T5" s="44"/>
-      <x:c r="U5" s="44"/>
-      <x:c r="V5" s="44"/>
-      <x:c r="W5" s="44"/>
+      <x:c r="A5" s="45"/>
+      <x:c r="B5" s="45"/>
+      <x:c r="C5" s="45"/>
+      <x:c r="D5" s="45"/>
+      <x:c r="E5" s="45"/>
+      <x:c r="F5" s="45"/>
+      <x:c r="G5" s="45"/>
+      <x:c r="H5" s="45"/>
+      <x:c r="I5" s="45"/>
+      <x:c r="J5" s="45"/>
+      <x:c r="K5" s="45"/>
+      <x:c r="L5" s="45"/>
+      <x:c r="M5" s="45"/>
+      <x:c r="N5" s="45"/>
+      <x:c r="O5" s="45"/>
+      <x:c r="P5" s="45"/>
+      <x:c r="Q5" s="45"/>
+      <x:c r="R5" s="45"/>
+      <x:c r="S5" s="45"/>
+      <x:c r="T5" s="45"/>
+      <x:c r="U5" s="45"/>
+      <x:c r="V5" s="45"/>
+      <x:c r="W5" s="45"/>
+      <x:c r="X5" s="45"/>
+      <x:c r="Y5" s="45"/>
+      <x:c r="Z5" s="45"/>
+      <x:c r="AA5" s="45"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="36" t="str">
+      <x:c r="A6" s="37" t="str">
         <x:v>Mes</x:v>
       </x:c>
-      <x:c r="B6" s="36" t="str">
+      <x:c r="B6" s="37" t="str">
         <x:v>Fecha</x:v>
       </x:c>
-      <x:c r="C6" s="36" t="str">
+      <x:c r="C6" s="37" t="str">
         <x:v>Chile base cloud</x:v>
       </x:c>
-      <x:c r="D6" s="36" t="str">
+      <x:c r="D6" s="37" t="str">
         <x:v>Chile optimizado cloud</x:v>
       </x:c>
-      <x:c r="E6" s="36" t="str">
+      <x:c r="E6" s="37" t="str">
         <x:v>Chile ahorro bruto</x:v>
       </x:c>
-      <x:c r="F6" s="36" t="str">
+      <x:c r="F6" s="37" t="str">
         <x:v>Chile operación</x:v>
       </x:c>
-      <x:c r="G6" s="36" t="str">
+      <x:c r="G6" s="37" t="str">
         <x:v>Chile CF cloud base</x:v>
       </x:c>
-      <x:c r="H6" s="36" t="str">
+      <x:c r="H6" s="37" t="str">
         <x:v>Chile CF cloud optimizado</x:v>
       </x:c>
-      <x:c r="I6" s="36" t="str">
+      <x:c r="I6" s="37" t="str">
         <x:v>Chile CF incremental</x:v>
       </x:c>
-      <x:c r="J6" s="36" t="str">
+      <x:c r="J6" s="37" t="str">
         <x:v>Chile CF económico optimizado</x:v>
       </x:c>
-      <x:c r="K6" s="36" t="str">
+      <x:c r="K6" s="37" t="str">
         <x:v>East base cloud</x:v>
       </x:c>
-      <x:c r="L6" s="36" t="str">
+      <x:c r="L6" s="37" t="str">
         <x:v>East optimizado cloud</x:v>
       </x:c>
-      <x:c r="M6" s="36" t="str">
+      <x:c r="M6" s="37" t="str">
         <x:v>East ahorro bruto</x:v>
       </x:c>
-      <x:c r="N6" s="36" t="str">
+      <x:c r="N6" s="37" t="str">
         <x:v>East operación</x:v>
       </x:c>
-      <x:c r="O6" s="36" t="str">
+      <x:c r="O6" s="37" t="str">
         <x:v>East CF cloud base</x:v>
       </x:c>
-      <x:c r="P6" s="36" t="str">
+      <x:c r="P6" s="37" t="str">
         <x:v>East CF cloud optimizado</x:v>
       </x:c>
-      <x:c r="Q6" s="36" t="str">
+      <x:c r="Q6" s="37" t="str">
         <x:v>East CF incremental</x:v>
       </x:c>
-      <x:c r="R6" s="36" t="str">
+      <x:c r="R6" s="37" t="str">
         <x:v>East CF económico optimizado</x:v>
       </x:c>
-      <x:c r="S6" s="36" t="str">
+      <x:c r="S6" s="37" t="str">
         <x:v>Factor descuento</x:v>
       </x:c>
-      <x:c r="T6" s="36" t="str">
+      <x:c r="T6" s="37" t="str">
         <x:v>Chile PV ahorro bruto</x:v>
       </x:c>
-      <x:c r="U6" s="36" t="str">
+      <x:c r="U6" s="37" t="str">
         <x:v>East PV ahorro bruto</x:v>
       </x:c>
-      <x:c r="V6" s="36" t="str">
+      <x:c r="V6" s="37" t="str">
         <x:v>Chile PV neto incremental</x:v>
       </x:c>
-      <x:c r="W6" s="36" t="str">
+      <x:c r="W6" s="37" t="str">
         <x:v>East PV neto incremental</x:v>
       </x:c>
+      <x:c r="X6" s="37" t="str">
+        <x:v>Chile PV neto acumulado</x:v>
+      </x:c>
+      <x:c r="Y6" s="37" t="str">
+        <x:v>East PV neto acumulado</x:v>
+      </x:c>
+      <x:c r="Z6" s="37" t="str">
+        <x:v>Chile mes recuperación</x:v>
+      </x:c>
+      <x:c r="AA6" s="37" t="str">
+        <x:v>East mes recuperación</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="29" t="n">
+      <x:c r="A7" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B7" s="28" t="n">
+      <x:c r="B7" s="29" t="n">
         <x:v>46023</x:v>
       </x:c>
       <x:c r="C7" s="12" t="n">
@@ -1580,7 +1640,7 @@
       <x:c r="R7" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(Supuestos!$B$12+Supuestos!$B$16))</x:f>
       </x:c>
-      <x:c r="S7" s="30" t="n">
+      <x:c r="S7" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A7</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -1598,12 +1658,26 @@
         <x:f>IF(Q7="","",Q7*S7)</x:f>
         <x:v>-426.72630819983806</x:v>
       </x:c>
+      <x:c r="X7" s="12" t="n">
+        <x:f>V7</x:f>
+        <x:v>-426.72630819983806</x:v>
+      </x:c>
+      <x:c r="Y7" s="12" t="n">
+        <x:f>W7</x:f>
+        <x:v>-426.72630819983806</x:v>
+      </x:c>
+      <x:c r="Z7" s="30" t="str">
+        <x:f>IF(X7&gt;=0,A7,"")</x:f>
+      </x:c>
+      <x:c r="AA7" s="30" t="str">
+        <x:f>IF(Y7&gt;=0,A7,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="29" t="n">
+      <x:c r="A8" s="30" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B8" s="28" t="n">
+      <x:c r="B8" s="29" t="n">
         <x:v>46054</x:v>
       </x:c>
       <x:c r="C8" s="12" t="n">
@@ -1668,7 +1742,7 @@
       <x:c r="R8" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L8+N8))</x:f>
       </x:c>
-      <x:c r="S8" s="30" t="n">
+      <x:c r="S8" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A8</x:f>
         <x:v>0.9955482081557259</x:v>
       </x:c>
@@ -1688,12 +1762,26 @@
         <x:f>IF(Q8="","",Q8*S8)</x:f>
         <x:v>7.041984202869434</x:v>
       </x:c>
+      <x:c r="X8" s="12" t="n">
+        <x:f>IF(V8="","",X7+V8)</x:f>
+        <x:v>-411.111459266898</x:v>
+      </x:c>
+      <x:c r="Y8" s="12" t="n">
+        <x:f>IF(W8="","",Y7+W8)</x:f>
+        <x:v>-419.6843239969686</x:v>
+      </x:c>
+      <x:c r="Z8" s="30" t="str">
+        <x:f>IF(AND(X8&gt;=0,X7&lt;0),A8,"")</x:f>
+      </x:c>
+      <x:c r="AA8" s="30" t="str">
+        <x:f>IF(AND(Y8&gt;=0,Y7&lt;0),A8,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="29" t="n">
+      <x:c r="A9" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="n">
+      <x:c r="B9" s="29" t="n">
         <x:v>46082</x:v>
       </x:c>
       <x:c r="C9" s="12" t="n">
@@ -1758,7 +1846,7 @@
       <x:c r="R9" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L9+N9))</x:f>
       </x:c>
-      <x:c r="S9" s="30" t="n">
+      <x:c r="S9" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A9</x:f>
         <x:v>0.9911162347620767</x:v>
       </x:c>
@@ -1778,12 +1866,26 @@
         <x:f>IF(Q9="","",Q9*S9)</x:f>
         <x:v>7.010634755027594</x:v>
       </x:c>
+      <x:c r="X9" s="12" t="n">
+        <x:f>IF(V9="","",X8+V9)</x:f>
+        <x:v>-395.5661243910872</x:v>
+      </x:c>
+      <x:c r="Y9" s="12" t="n">
+        <x:f>IF(W9="","",Y8+W9)</x:f>
+        <x:v>-412.673689241941</x:v>
+      </x:c>
+      <x:c r="Z9" s="30" t="str">
+        <x:f>IF(AND(X9&gt;=0,X8&lt;0),A9,"")</x:f>
+      </x:c>
+      <x:c r="AA9" s="30" t="str">
+        <x:f>IF(AND(Y9&gt;=0,Y8&lt;0),A9,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="29" t="n">
+      <x:c r="A10" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="n">
+      <x:c r="B10" s="29" t="n">
         <x:v>46113</x:v>
       </x:c>
       <x:c r="C10" s="12" t="n">
@@ -1848,7 +1950,7 @@
       <x:c r="R10" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L10+N10))</x:f>
       </x:c>
-      <x:c r="S10" s="30" t="n">
+      <x:c r="S10" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A10</x:f>
         <x:v>0.9867039915914352</x:v>
       </x:c>
@@ -1868,12 +1970,26 @@
         <x:f>IF(Q10="","",Q10*S10)</x:f>
         <x:v>6.979424868401978</x:v>
       </x:c>
+      <x:c r="X10" s="12" t="n">
+        <x:f>IF(V10="","",X9+V10)</x:f>
+        <x:v>-380.08999411029305</x:v>
+      </x:c>
+      <x:c r="Y10" s="12" t="n">
+        <x:f>IF(W10="","",Y9+W10)</x:f>
+        <x:v>-405.69426437353906</x:v>
+      </x:c>
+      <x:c r="Z10" s="30" t="str">
+        <x:f>IF(AND(X10&gt;=0,X9&lt;0),A10,"")</x:f>
+      </x:c>
+      <x:c r="AA10" s="30" t="str">
+        <x:f>IF(AND(Y10&gt;=0,Y9&lt;0),A10,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="29" t="n">
+      <x:c r="A11" s="30" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
+      <x:c r="B11" s="29" t="n">
         <x:v>46143</x:v>
       </x:c>
       <x:c r="C11" s="12" t="n">
@@ -1938,7 +2054,7 @@
       <x:c r="R11" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L11+N11))</x:f>
       </x:c>
-      <x:c r="S11" s="30" t="n">
+      <x:c r="S11" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A11</x:f>
         <x:v>0.9823113908089557</x:v>
       </x:c>
@@ -1958,12 +2074,26 @@
         <x:f>IF(Q11="","",Q11*S11)</x:f>
         <x:v>6.948353921695102</x:v>
       </x:c>
+      <x:c r="X11" s="12" t="n">
+        <x:f>IF(V11="","",X10+V11)</x:f>
+        <x:v>-364.68276034006385</x:v>
+      </x:c>
+      <x:c r="Y11" s="12" t="n">
+        <x:f>IF(W11="","",Y10+W11)</x:f>
+        <x:v>-398.74591045184394</x:v>
+      </x:c>
+      <x:c r="Z11" s="30" t="str">
+        <x:f>IF(AND(X11&gt;=0,X10&lt;0),A11,"")</x:f>
+      </x:c>
+      <x:c r="AA11" s="30" t="str">
+        <x:f>IF(AND(Y11&gt;=0,Y10&lt;0),A11,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="29" t="n">
+      <x:c r="A12" s="30" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B12" s="28" t="n">
+      <x:c r="B12" s="29" t="n">
         <x:v>46174</x:v>
       </x:c>
       <x:c r="C12" s="12" t="n">
@@ -2028,7 +2158,7 @@
       <x:c r="R12" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L12+N12))</x:f>
       </x:c>
-      <x:c r="S12" s="30" t="n">
+      <x:c r="S12" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A12</x:f>
         <x:v>0.9779383449708149</x:v>
       </x:c>
@@ -2048,12 +2178,26 @@
         <x:f>IF(Q12="","",Q12*S12)</x:f>
         <x:v>6.91742129637537</x:v>
       </x:c>
+      <x:c r="X12" s="12" t="n">
+        <x:f>IF(V12="","",X11+V12)</x:f>
+        <x:v>-349.3441163674758</x:v>
+      </x:c>
+      <x:c r="Y12" s="12" t="n">
+        <x:f>IF(W12="","",Y11+W12)</x:f>
+        <x:v>-391.82848915546856</x:v>
+      </x:c>
+      <x:c r="Z12" s="30" t="str">
+        <x:f>IF(AND(X12&gt;=0,X11&lt;0),A12,"")</x:f>
+      </x:c>
+      <x:c r="AA12" s="30" t="str">
+        <x:f>IF(AND(Y12&gt;=0,Y11&lt;0),A12,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="29" t="n">
+      <x:c r="A13" s="30" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B13" s="28" t="n">
+      <x:c r="B13" s="29" t="n">
         <x:v>46204</x:v>
       </x:c>
       <x:c r="C13" s="12" t="n">
@@ -2118,7 +2262,7 @@
       <x:c r="R13" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L13+N13))</x:f>
       </x:c>
-      <x:c r="S13" s="30" t="n">
+      <x:c r="S13" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A13</x:f>
         <x:v>0.973584767022471</x:v>
       </x:c>
@@ -2138,12 +2282,26 @@
         <x:f>IF(Q13="","",Q13*S13)</x:f>
         <x:v>6.886626376664759</x:v>
       </x:c>
+      <x:c r="X13" s="12" t="n">
+        <x:f>IF(V13="","",X12+V13)</x:f>
+        <x:v>-334.07375684502716</x:v>
+      </x:c>
+      <x:c r="Y13" s="12" t="n">
+        <x:f>IF(W13="","",Y12+W13)</x:f>
+        <x:v>-384.9418627788038</x:v>
+      </x:c>
+      <x:c r="Z13" s="30" t="str">
+        <x:f>IF(AND(X13&gt;=0,X12&lt;0),A13,"")</x:f>
+      </x:c>
+      <x:c r="AA13" s="30" t="str">
+        <x:f>IF(AND(Y13&gt;=0,Y12&lt;0),A13,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="29" t="n">
+      <x:c r="A14" s="30" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B14" s="28" t="n">
+      <x:c r="B14" s="29" t="n">
         <x:v>46235</x:v>
       </x:c>
       <x:c r="C14" s="12" t="n">
@@ -2208,7 +2366,7 @@
       <x:c r="R14" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L14+N14))</x:f>
       </x:c>
-      <x:c r="S14" s="30" t="n">
+      <x:c r="S14" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A14</x:f>
         <x:v>0.9692505702969308</x:v>
       </x:c>
@@ -2228,12 +2386,26 @@
         <x:f>IF(Q14="","",Q14*S14)</x:f>
         <x:v>6.855968549526559</x:v>
       </x:c>
+      <x:c r="X14" s="12" t="n">
+        <x:f>IF(V14="","",X13+V14)</x:f>
+        <x:v>-318.8713777845597</x:v>
+      </x:c>
+      <x:c r="Y14" s="12" t="n">
+        <x:f>IF(W14="","",Y13+W14)</x:f>
+        <x:v>-378.08589422927724</x:v>
+      </x:c>
+      <x:c r="Z14" s="30" t="str">
+        <x:f>IF(AND(X14&gt;=0,X13&lt;0),A14,"")</x:f>
+      </x:c>
+      <x:c r="AA14" s="30" t="str">
+        <x:f>IF(AND(Y14&gt;=0,Y13&lt;0),A14,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="29" t="n">
+      <x:c r="A15" s="30" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B15" s="28" t="n">
+      <x:c r="B15" s="29" t="n">
         <x:v>46266</x:v>
       </x:c>
       <x:c r="C15" s="12" t="n">
@@ -2298,7 +2470,7 @@
       <x:c r="R15" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L15+N15))</x:f>
       </x:c>
-      <x:c r="S15" s="30" t="n">
+      <x:c r="S15" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A15</x:f>
         <x:v>0.964935668513025</x:v>
       </x:c>
@@ -2318,12 +2490,26 @@
         <x:f>IF(Q15="","",Q15*S15)</x:f>
         <x:v>6.825447204653178</x:v>
       </x:c>
+      <x:c r="X15" s="12" t="n">
+        <x:f>IF(V15="","",X14+V15)</x:f>
+        <x:v>-303.73667655120715</x:v>
+      </x:c>
+      <x:c r="Y15" s="12" t="n">
+        <x:f>IF(W15="","",Y14+W15)</x:f>
+        <x:v>-371.26044702462406</x:v>
+      </x:c>
+      <x:c r="Z15" s="30" t="str">
+        <x:f>IF(AND(X15&gt;=0,X14&lt;0),A15,"")</x:f>
+      </x:c>
+      <x:c r="AA15" s="30" t="str">
+        <x:f>IF(AND(Y15&gt;=0,Y14&lt;0),A15,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29" t="n">
+      <x:c r="A16" s="30" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
+      <x:c r="B16" s="29" t="n">
         <x:v>46296</x:v>
       </x:c>
       <x:c r="C16" s="12" t="n">
@@ -2388,7 +2574,7 @@
       <x:c r="R16" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L16+N16))</x:f>
       </x:c>
-      <x:c r="S16" s="30" t="n">
+      <x:c r="S16" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A16</x:f>
         <x:v>0.9606399757736895</x:v>
       </x:c>
@@ -2408,12 +2594,26 @@
         <x:f>IF(Q16="","",Q16*S16)</x:f>
         <x:v>6.795061734453979</x:v>
       </x:c>
+      <x:c r="X16" s="12" t="n">
+        <x:f>IF(V16="","",X15+V16)</x:f>
+        <x:v>-288.66935185737077</x:v>
+      </x:c>
+      <x:c r="Y16" s="12" t="n">
+        <x:f>IF(W16="","",Y15+W16)</x:f>
+        <x:v>-364.4653852901701</x:v>
+      </x:c>
+      <x:c r="Z16" s="30" t="str">
+        <x:f>IF(AND(X16&gt;=0,X15&lt;0),A16,"")</x:f>
+      </x:c>
+      <x:c r="AA16" s="30" t="str">
+        <x:f>IF(AND(Y16&gt;=0,Y15&lt;0),A16,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="n">
+      <x:c r="A17" s="30" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B17" s="28" t="n">
+      <x:c r="B17" s="29" t="n">
         <x:v>46327</x:v>
       </x:c>
       <x:c r="C17" s="12" t="n">
@@ -2478,7 +2678,7 @@
       <x:c r="R17" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L17+N17))</x:f>
       </x:c>
-      <x:c r="S17" s="30" t="n">
+      <x:c r="S17" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A17</x:f>
         <x:v>0.9563634065642566</x:v>
       </x:c>
@@ -2498,12 +2698,26 @@
         <x:f>IF(Q17="","",Q17*S17)</x:f>
         <x:v>6.764811534043198</x:v>
       </x:c>
+      <x:c r="X17" s="12" t="n">
+        <x:f>IF(V17="","",X16+V17)</x:f>
+        <x:v>-273.6691037567214</x:v>
+      </x:c>
+      <x:c r="Y17" s="12" t="n">
+        <x:f>IF(W17="","",Y16+W17)</x:f>
+        <x:v>-357.7005737561269</x:v>
+      </x:c>
+      <x:c r="Z17" s="30" t="str">
+        <x:f>IF(AND(X17&gt;=0,X16&lt;0),A17,"")</x:f>
+      </x:c>
+      <x:c r="AA17" s="30" t="str">
+        <x:f>IF(AND(Y17&gt;=0,Y16&lt;0),A17,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="29" t="n">
+      <x:c r="A18" s="30" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B18" s="28" t="n">
+      <x:c r="B18" s="29" t="n">
         <x:v>46357</x:v>
       </x:c>
       <x:c r="C18" s="12" t="n">
@@ -2568,7 +2782,7 @@
       <x:c r="R18" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L18+N18))</x:f>
       </x:c>
-      <x:c r="S18" s="30" t="n">
+      <x:c r="S18" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A18</x:f>
         <x:v>0.9521058757507516</x:v>
       </x:c>
@@ -2588,12 +2802,26 @@
         <x:f>IF(Q18="","",Q18*S18)</x:f>
         <x:v>6.734696001227893</x:v>
       </x:c>
+      <x:c r="X18" s="12" t="n">
+        <x:f>IF(V18="","",X17+V18)</x:f>
+        <x:v>-258.73563363822865</x:v>
+      </x:c>
+      <x:c r="Y18" s="12" t="n">
+        <x:f>IF(W18="","",Y17+W18)</x:f>
+        <x:v>-350.965877754899</x:v>
+      </x:c>
+      <x:c r="Z18" s="30" t="str">
+        <x:f>IF(AND(X18&gt;=0,X17&lt;0),A18,"")</x:f>
+      </x:c>
+      <x:c r="AA18" s="30" t="str">
+        <x:f>IF(AND(Y18&gt;=0,Y17&lt;0),A18,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="29" t="n">
+      <x:c r="A19" s="30" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B19" s="28" t="n">
+      <x:c r="B19" s="29" t="n">
         <x:v>46388</x:v>
       </x:c>
       <x:c r="C19" s="12" t="n">
@@ -2658,7 +2886,7 @@
       <x:c r="R19" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L19+N19))</x:f>
       </x:c>
-      <x:c r="S19" s="30" t="n">
+      <x:c r="S19" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A19</x:f>
         <x:v>0.947867298578199</x:v>
       </x:c>
@@ -2678,12 +2906,26 @@
         <x:f>IF(Q19="","",Q19*S19)</x:f>
         <x:v>6.7047145364959615</x:v>
       </x:c>
+      <x:c r="X19" s="12" t="n">
+        <x:f>IF(V19="","",X18+V19)</x:f>
+        <x:v>-243.8686442202161</x:v>
+      </x:c>
+      <x:c r="Y19" s="12" t="n">
+        <x:f>IF(W19="","",Y18+W19)</x:f>
+        <x:v>-344.26116321840306</x:v>
+      </x:c>
+      <x:c r="Z19" s="30" t="str">
+        <x:f>IF(AND(X19&gt;=0,X18&lt;0),A19,"")</x:f>
+      </x:c>
+      <x:c r="AA19" s="30" t="str">
+        <x:f>IF(AND(Y19&gt;=0,Y18&lt;0),A19,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="29" t="n">
+      <x:c r="A20" s="30" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B20" s="28" t="n">
+      <x:c r="B20" s="29" t="n">
         <x:v>46419</x:v>
       </x:c>
       <x:c r="C20" s="12" t="n">
@@ -2748,7 +2990,7 @@
       <x:c r="R20" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L20+N20))</x:f>
       </x:c>
-      <x:c r="S20" s="30" t="n">
+      <x:c r="S20" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A20</x:f>
         <x:v>0.9436475906689343</x:v>
       </x:c>
@@ -2768,12 +3010,26 @@
         <x:f>IF(Q20="","",Q20*S20)</x:f>
         <x:v>6.674866543004202</x:v>
       </x:c>
+      <x:c r="X20" s="12" t="n">
+        <x:f>IF(V20="","",X19+V20)</x:f>
+        <x:v>-229.0678395444436</x:v>
+      </x:c>
+      <x:c r="Y20" s="12" t="n">
+        <x:f>IF(W20="","",Y19+W20)</x:f>
+        <x:v>-337.58629667539884</x:v>
+      </x:c>
+      <x:c r="Z20" s="30" t="str">
+        <x:f>IF(AND(X20&gt;=0,X19&lt;0),A20,"")</x:f>
+      </x:c>
+      <x:c r="AA20" s="30" t="str">
+        <x:f>IF(AND(Y20&gt;=0,Y19&lt;0),A20,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="29" t="n">
+      <x:c r="A21" s="30" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B21" s="28" t="n">
+      <x:c r="B21" s="29" t="n">
         <x:v>46447</x:v>
       </x:c>
       <x:c r="C21" s="12" t="n">
@@ -2838,7 +3094,7 @@
       <x:c r="R21" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L21+N21))</x:f>
       </x:c>
-      <x:c r="S21" s="30" t="n">
+      <x:c r="S21" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A21</x:f>
         <x:v>0.9394466680209257</x:v>
       </x:c>
@@ -2858,12 +3114,26 @@
         <x:f>IF(Q21="","",Q21*S21)</x:f>
         <x:v>6.645151426566439</x:v>
       </x:c>
+      <x:c r="X21" s="12" t="n">
+        <x:f>IF(V21="","",X20+V21)</x:f>
+        <x:v>-214.33292497021534</x:v>
+      </x:c>
+      <x:c r="Y21" s="12" t="n">
+        <x:f>IF(W21="","",Y20+W21)</x:f>
+        <x:v>-330.9411452488324</x:v>
+      </x:c>
+      <x:c r="Z21" s="30" t="str">
+        <x:f>IF(AND(X21&gt;=0,X20&lt;0),A21,"")</x:f>
+      </x:c>
+      <x:c r="AA21" s="30" t="str">
+        <x:f>IF(AND(Y21&gt;=0,Y20&lt;0),A21,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="29" t="n">
+      <x:c r="A22" s="30" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B22" s="28" t="n">
+      <x:c r="B22" s="29" t="n">
         <x:v>46478</x:v>
       </x:c>
       <x:c r="C22" s="12" t="n">
@@ -2928,7 +3198,7 @@
       <x:c r="R22" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L22+N22))</x:f>
       </x:c>
-      <x:c r="S22" s="30" t="n">
+      <x:c r="S22" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A22</x:f>
         <x:v>0.9352644470060996</x:v>
       </x:c>
@@ -2948,12 +3218,26 @@
         <x:f>IF(Q22="","",Q22*S22)</x:f>
         <x:v>6.615568595641684</x:v>
       </x:c>
+      <x:c r="X22" s="12" t="n">
+        <x:f>IF(V22="","",X21+V22)</x:f>
+        <x:v>-199.66360716851474</x:v>
+      </x:c>
+      <x:c r="Y22" s="12" t="n">
+        <x:f>IF(W22="","",Y21+W22)</x:f>
+        <x:v>-324.32557665319075</x:v>
+      </x:c>
+      <x:c r="Z22" s="30" t="str">
+        <x:f>IF(AND(X22&gt;=0,X21&lt;0),A22,"")</x:f>
+      </x:c>
+      <x:c r="AA22" s="30" t="str">
+        <x:f>IF(AND(Y22&gt;=0,Y21&lt;0),A22,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="29" t="n">
+      <x:c r="A23" s="30" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B23" s="28" t="n">
+      <x:c r="B23" s="29" t="n">
         <x:v>46508</x:v>
       </x:c>
       <x:c r="C23" s="12" t="n">
@@ -3018,7 +3302,7 @@
       <x:c r="R23" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L23+N23))</x:f>
       </x:c>
-      <x:c r="S23" s="30" t="n">
+      <x:c r="S23" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A23</x:f>
         <x:v>0.9311008443686783</x:v>
       </x:c>
@@ -3038,12 +3322,26 @@
         <x:f>IF(Q23="","",Q23*S23)</x:f>
         <x:v>6.586117461322371</x:v>
       </x:c>
+      <x:c r="X23" s="12" t="n">
+        <x:f>IF(V23="","",X22+V23)</x:f>
+        <x:v>-185.05959411616482</x:v>
+      </x:c>
+      <x:c r="Y23" s="12" t="n">
+        <x:f>IF(W23="","",Y22+W23)</x:f>
+        <x:v>-317.7394591918684</x:v>
+      </x:c>
+      <x:c r="Z23" s="30" t="str">
+        <x:f>IF(AND(X23&gt;=0,X22&lt;0),A23,"")</x:f>
+      </x:c>
+      <x:c r="AA23" s="30" t="str">
+        <x:f>IF(AND(Y23&gt;=0,Y22&lt;0),A23,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="29" t="n">
+      <x:c r="A24" s="30" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B24" s="28" t="n">
+      <x:c r="B24" s="29" t="n">
         <x:v>46539</x:v>
       </x:c>
       <x:c r="C24" s="12" t="n">
@@ -3108,7 +3406,7 @@
       <x:c r="R24" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L24+N24))</x:f>
       </x:c>
-      <x:c r="S24" s="30" t="n">
+      <x:c r="S24" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A24</x:f>
         <x:v>0.9269557772235212</x:v>
       </x:c>
@@ -3128,12 +3426,26 @@
         <x:f>IF(Q24="","",Q24*S24)</x:f>
         <x:v>6.556797437322625</x:v>
       </x:c>
+      <x:c r="X24" s="12" t="n">
+        <x:f>IF(V24="","",X23+V24)</x:f>
+        <x:v>-170.520595090015</x:v>
+      </x:c>
+      <x:c r="Y24" s="12" t="n">
+        <x:f>IF(W24="","",Y23+W24)</x:f>
+        <x:v>-311.18266175454573</x:v>
+      </x:c>
+      <x:c r="Z24" s="30" t="str">
+        <x:f>IF(AND(X24&gt;=0,X23&lt;0),A24,"")</x:f>
+      </x:c>
+      <x:c r="AA24" s="30" t="str">
+        <x:f>IF(AND(Y24&gt;=0,Y23&lt;0),A24,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="29" t="n">
+      <x:c r="A25" s="30" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B25" s="28" t="n">
+      <x:c r="B25" s="29" t="n">
         <x:v>46569</x:v>
       </x:c>
       <x:c r="C25" s="12" t="n">
@@ -3198,7 +3510,7 @@
       <x:c r="R25" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L25+N25))</x:f>
       </x:c>
-      <x:c r="S25" s="30" t="n">
+      <x:c r="S25" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A25</x:f>
         <x:v>0.9228291630544746</x:v>
       </x:c>
@@ -3218,12 +3530,26 @@
         <x:f>IF(Q25="","",Q25*S25)</x:f>
         <x:v>6.527607939966594</x:v>
       </x:c>
+      <x:c r="X25" s="12" t="n">
+        <x:f>IF(V25="","",X24+V25)</x:f>
+        <x:v>-156.04632066115371</x:v>
+      </x:c>
+      <x:c r="Y25" s="12" t="n">
+        <x:f>IF(W25="","",Y24+W25)</x:f>
+        <x:v>-304.65505381457916</x:v>
+      </x:c>
+      <x:c r="Z25" s="30" t="str">
+        <x:f>IF(AND(X25&gt;=0,X24&lt;0),A25,"")</x:f>
+      </x:c>
+      <x:c r="AA25" s="30" t="str">
+        <x:f>IF(AND(Y25&gt;=0,Y24&lt;0),A25,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="29" t="n">
+      <x:c r="A26" s="30" t="n">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B26" s="28" t="n">
+      <x:c r="B26" s="29" t="n">
         <x:v>46600</x:v>
       </x:c>
       <x:c r="C26" s="12" t="n">
@@ -3288,7 +3614,7 @@
       <x:c r="R26" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L26+N26))</x:f>
       </x:c>
-      <x:c r="S26" s="30" t="n">
+      <x:c r="S26" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A26</x:f>
         <x:v>0.9187209197127305</x:v>
       </x:c>
@@ -3308,12 +3634,26 @@
         <x:f>IF(Q26="","",Q26*S26)</x:f>
         <x:v>6.4985483881768324</x:v>
       </x:c>
+      <x:c r="X26" s="12" t="n">
+        <x:f>IF(V26="","",X25+V26)</x:f>
+        <x:v>-141.63648268914662</x:v>
+      </x:c>
+      <x:c r="Y26" s="12" t="n">
+        <x:f>IF(W26="","",Y25+W26)</x:f>
+        <x:v>-298.1565054264023</x:v>
+      </x:c>
+      <x:c r="Z26" s="30" t="str">
+        <x:f>IF(AND(X26&gt;=0,X25&lt;0),A26,"")</x:f>
+      </x:c>
+      <x:c r="AA26" s="30" t="str">
+        <x:f>IF(AND(Y26&gt;=0,Y25&lt;0),A26,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="29" t="n">
+      <x:c r="A27" s="30" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B27" s="28" t="n">
+      <x:c r="B27" s="29" t="n">
         <x:v>46631</x:v>
       </x:c>
       <x:c r="C27" s="12" t="n">
@@ -3378,7 +3718,7 @@
       <x:c r="R27" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L27+N27))</x:f>
       </x:c>
-      <x:c r="S27" s="30" t="n">
+      <x:c r="S27" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A27</x:f>
         <x:v>0.9146309654151893</x:v>
       </x:c>
@@ -3398,12 +3738,26 @@
         <x:f>IF(Q27="","",Q27*S27)</x:f>
         <x:v>6.469618203462725</x:v>
       </x:c>
+      <x:c r="X27" s="12" t="n">
+        <x:f>IF(V27="","",X26+V27)</x:f>
+        <x:v>-127.29079431630062</x:v>
+      </x:c>
+      <x:c r="Y27" s="12" t="n">
+        <x:f>IF(W27="","",Y26+W27)</x:f>
+        <x:v>-291.68688722293956</x:v>
+      </x:c>
+      <x:c r="Z27" s="30" t="str">
+        <x:f>IF(AND(X27&gt;=0,X26&lt;0),A27,"")</x:f>
+      </x:c>
+      <x:c r="AA27" s="30" t="str">
+        <x:f>IF(AND(Y27&gt;=0,Y26&lt;0),A27,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="29" t="n">
+      <x:c r="A28" s="30" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B28" s="28" t="n">
+      <x:c r="B28" s="29" t="n">
         <x:v>46661</x:v>
       </x:c>
       <x:c r="C28" s="12" t="n">
@@ -3468,7 +3822,7 @@
       <x:c r="R28" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L28+N28))</x:f>
       </x:c>
-      <x:c r="S28" s="30" t="n">
+      <x:c r="S28" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A28</x:f>
         <x:v>0.9105592187428335</x:v>
       </x:c>
@@ -3488,12 +3842,26 @@
         <x:f>IF(Q28="","",Q28*S28)</x:f>
         <x:v>6.440816809908984</x:v>
       </x:c>
+      <x:c r="X28" s="12" t="n">
+        <x:f>IF(V28="","",X27+V28)</x:f>
+        <x:v>-113.00896996195334</x:v>
+      </x:c>
+      <x:c r="Y28" s="12" t="n">
+        <x:f>IF(W28="","",Y27+W28)</x:f>
+        <x:v>-285.24607041303057</x:v>
+      </x:c>
+      <x:c r="Z28" s="30" t="str">
+        <x:f>IF(AND(X28&gt;=0,X27&lt;0),A28,"")</x:f>
+      </x:c>
+      <x:c r="AA28" s="30" t="str">
+        <x:f>IF(AND(Y28&gt;=0,Y27&lt;0),A28,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="29" t="n">
+      <x:c r="A29" s="30" t="n">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B29" s="28" t="n">
+      <x:c r="B29" s="29" t="n">
         <x:v>46692</x:v>
       </x:c>
       <x:c r="C29" s="12" t="n">
@@ -3558,7 +3926,7 @@
       <x:c r="R29" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L29+N29))</x:f>
       </x:c>
-      <x:c r="S29" s="30" t="n">
+      <x:c r="S29" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A29</x:f>
         <x:v>0.9065055986391056</x:v>
       </x:c>
@@ -3578,12 +3946,26 @@
         <x:f>IF(Q29="","",Q29*S29)</x:f>
         <x:v>6.412143634164168</x:v>
       </x:c>
+      <x:c r="X29" s="12" t="n">
+        <x:f>IF(V29="","",X28+V29)</x:f>
+        <x:v>-98.79072531678811</x:v>
+      </x:c>
+      <x:c r="Y29" s="12" t="n">
+        <x:f>IF(W29="","",Y28+W29)</x:f>
+        <x:v>-278.8339267788664</x:v>
+      </x:c>
+      <x:c r="Z29" s="30" t="str">
+        <x:f>IF(AND(X29&gt;=0,X28&lt;0),A29,"")</x:f>
+      </x:c>
+      <x:c r="AA29" s="30" t="str">
+        <x:f>IF(AND(Y29&gt;=0,Y28&lt;0),A29,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="29" t="n">
+      <x:c r="A30" s="30" t="n">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B30" s="28" t="n">
+      <x:c r="B30" s="29" t="n">
         <x:v>46722</x:v>
       </x:c>
       <x:c r="C30" s="12" t="n">
@@ -3648,7 +4030,7 @@
       <x:c r="R30" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L30+N30))</x:f>
       </x:c>
-      <x:c r="S30" s="30" t="n">
+      <x:c r="S30" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A30</x:f>
         <x:v>0.9024700244082953</x:v>
       </x:c>
@@ -3668,12 +4050,26 @@
         <x:f>IF(Q30="","",Q30*S30)</x:f>
         <x:v>6.383598105429281</x:v>
       </x:c>
+      <x:c r="X30" s="12" t="n">
+        <x:f>IF(V30="","",X29+V30)</x:f>
+        <x:v>-84.63577733717412</x:v>
+      </x:c>
+      <x:c r="Y30" s="12" t="n">
+        <x:f>IF(W30="","",Y29+W30)</x:f>
+        <x:v>-272.4503286734371</x:v>
+      </x:c>
+      <x:c r="Z30" s="30" t="str">
+        <x:f>IF(AND(X30&gt;=0,X29&lt;0),A30,"")</x:f>
+      </x:c>
+      <x:c r="AA30" s="30" t="str">
+        <x:f>IF(AND(Y30&gt;=0,Y29&lt;0),A30,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="29" t="n">
+      <x:c r="A31" s="30" t="n">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B31" s="28" t="n">
+      <x:c r="B31" s="29" t="n">
         <x:v>46753</x:v>
       </x:c>
       <x:c r="C31" s="12" t="n">
@@ -3738,7 +4134,7 @@
       <x:c r="R31" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L31+N31))</x:f>
       </x:c>
-      <x:c r="S31" s="30" t="n">
+      <x:c r="S31" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A31</x:f>
         <x:v>0.8984524157139326</x:v>
       </x:c>
@@ -3758,12 +4154,26 @@
         <x:f>IF(Q31="","",Q31*S31)</x:f>
         <x:v>6.355179655446409</x:v>
       </x:c>
+      <x:c r="X31" s="12" t="n">
+        <x:f>IF(V31="","",X30+V31)</x:f>
+        <x:v>-70.5438442395319</x:v>
+      </x:c>
+      <x:c r="Y31" s="12" t="n">
+        <x:f>IF(W31="","",Y30+W31)</x:f>
+        <x:v>-266.0951490179907</x:v>
+      </x:c>
+      <x:c r="Z31" s="30" t="str">
+        <x:f>IF(AND(X31&gt;=0,X30&lt;0),A31,"")</x:f>
+      </x:c>
+      <x:c r="AA31" s="30" t="str">
+        <x:f>IF(AND(Y31&gt;=0,Y30&lt;0),A31,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="29" t="n">
+      <x:c r="A32" s="30" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B32" s="28" t="n">
+      <x:c r="B32" s="29" t="n">
         <x:v>46784</x:v>
       </x:c>
       <x:c r="C32" s="12" t="n">
@@ -3828,7 +4238,7 @@
       <x:c r="R32" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L32+N32))</x:f>
       </x:c>
-      <x:c r="S32" s="30" t="n">
+      <x:c r="S32" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A32</x:f>
         <x:v>0.894452692577189</x:v>
       </x:c>
@@ -3848,12 +4258,26 @@
         <x:f>IF(Q32="","",Q32*S32)</x:f>
         <x:v>6.326887718487395</x:v>
       </x:c>
+      <x:c r="X32" s="12" t="n">
+        <x:f>IF(V32="","",X31+V32)</x:f>
+        <x:v>-56.51464549472381</x:v>
+      </x:c>
+      <x:c r="Y32" s="12" t="n">
+        <x:f>IF(W32="","",Y31+W32)</x:f>
+        <x:v>-259.7682612995033</x:v>
+      </x:c>
+      <x:c r="Z32" s="30" t="str">
+        <x:f>IF(AND(X32&gt;=0,X31&lt;0),A32,"")</x:f>
+      </x:c>
+      <x:c r="AA32" s="30" t="str">
+        <x:f>IF(AND(Y32&gt;=0,Y31&lt;0),A32,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="29" t="n">
+      <x:c r="A33" s="30" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="B33" s="28" t="n">
+      <x:c r="B33" s="29" t="n">
         <x:v>46813</x:v>
       </x:c>
       <x:c r="C33" s="12" t="n">
@@ -3918,7 +4342,7 @@
       <x:c r="R33" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L33+N33))</x:f>
       </x:c>
-      <x:c r="S33" s="30" t="n">
+      <x:c r="S33" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A33</x:f>
         <x:v>0.8904707753752847</x:v>
       </x:c>
@@ -3938,12 +4362,26 @@
         <x:f>IF(Q33="","",Q33*S33)</x:f>
         <x:v>6.298721731342595</x:v>
       </x:c>
+      <x:c r="X33" s="12" t="n">
+        <x:f>IF(V33="","",X32+V33)</x:f>
+        <x:v>-42.54790182246956</x:v>
+      </x:c>
+      <x:c r="Y33" s="12" t="n">
+        <x:f>IF(W33="","",Y32+W33)</x:f>
+        <x:v>-253.4695395681607</x:v>
+      </x:c>
+      <x:c r="Z33" s="30" t="str">
+        <x:f>IF(AND(X33&gt;=0,X32&lt;0),A33,"")</x:f>
+      </x:c>
+      <x:c r="AA33" s="30" t="str">
+        <x:f>IF(AND(Y33&gt;=0,Y32&lt;0),A33,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="29" t="n">
+      <x:c r="A34" s="30" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B34" s="28" t="n">
+      <x:c r="B34" s="29" t="n">
         <x:v>46844</x:v>
       </x:c>
       <x:c r="C34" s="12" t="n">
@@ -4008,7 +4446,7 @@
       <x:c r="R34" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L34+N34))</x:f>
       </x:c>
-      <x:c r="S34" s="30" t="n">
+      <x:c r="S34" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A34</x:f>
         <x:v>0.8865065848399046</x:v>
       </x:c>
@@ -4028,12 +4466,26 @@
         <x:f>IF(Q34="","",Q34*S34)</x:f>
         <x:v>6.270681133309652</x:v>
       </x:c>
+      <x:c r="X34" s="12" t="n">
+        <x:f>IF(V34="","",X33+V34)</x:f>
+        <x:v>-28.643335185786523</x:v>
+      </x:c>
+      <x:c r="Y34" s="12" t="n">
+        <x:f>IF(W34="","",Y33+W34)</x:f>
+        <x:v>-247.19885843485105</x:v>
+      </x:c>
+      <x:c r="Z34" s="30" t="str">
+        <x:f>IF(AND(X34&gt;=0,X33&lt;0),A34,"")</x:f>
+      </x:c>
+      <x:c r="AA34" s="30" t="str">
+        <x:f>IF(AND(Y34&gt;=0,Y33&lt;0),A34,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="29" t="n">
+      <x:c r="A35" s="30" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B35" s="28" t="n">
+      <x:c r="B35" s="29" t="n">
         <x:v>46874</x:v>
       </x:c>
       <x:c r="C35" s="12" t="n">
@@ -4098,7 +4550,7 @@
       <x:c r="R35" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L35+N35))</x:f>
       </x:c>
-      <x:c r="S35" s="30" t="n">
+      <x:c r="S35" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A35</x:f>
         <x:v>0.8825600420556191</x:v>
       </x:c>
@@ -4118,12 +4570,26 @@
         <x:f>IF(Q35="","",Q35*S35)</x:f>
         <x:v>6.242765366182341</x:v>
       </x:c>
+      <x:c r="X35" s="12" t="n">
+        <x:f>IF(V35="","",X34+V35)</x:f>
+        <x:v>-14.800668785454834</x:v>
+      </x:c>
+      <x:c r="Y35" s="12" t="n">
+        <x:f>IF(W35="","",Y34+W35)</x:f>
+        <x:v>-240.9560930686687</x:v>
+      </x:c>
+      <x:c r="Z35" s="30" t="str">
+        <x:f>IF(AND(X35&gt;=0,X34&lt;0),A35,"")</x:f>
+      </x:c>
+      <x:c r="AA35" s="30" t="str">
+        <x:f>IF(AND(Y35&gt;=0,Y34&lt;0),A35,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="29" t="n">
+      <x:c r="A36" s="30" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B36" s="28" t="n">
+      <x:c r="B36" s="29" t="n">
         <x:v>46905</x:v>
       </x:c>
       <x:c r="C36" s="12" t="n">
@@ -4188,7 +4654,7 @@
       <x:c r="R36" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L36+N36))</x:f>
       </x:c>
-      <x:c r="S36" s="30" t="n">
+      <x:c r="S36" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A36</x:f>
         <x:v>0.8786310684583137</x:v>
       </x:c>
@@ -4208,12 +4674,26 @@
         <x:f>IF(Q36="","",Q36*S36)</x:f>
         <x:v>6.214973874239454</x:v>
       </x:c>
+      <x:c r="X36" s="12" t="n">
+        <x:f>IF(V36="","",X35+V36)</x:f>
+        <x:v>-1.0196270545071489</x:v>
+      </x:c>
+      <x:c r="Y36" s="12" t="n">
+        <x:f>IF(W36="","",Y35+W36)</x:f>
+        <x:v>-234.74111919442925</x:v>
+      </x:c>
+      <x:c r="Z36" s="30" t="str">
+        <x:f>IF(AND(X36&gt;=0,X35&lt;0),A36,"")</x:f>
+      </x:c>
+      <x:c r="AA36" s="30" t="str">
+        <x:f>IF(AND(Y36&gt;=0,Y35&lt;0),A36,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="29" t="n">
+      <x:c r="A37" s="30" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B37" s="28" t="n">
+      <x:c r="B37" s="29" t="n">
         <x:v>46935</x:v>
       </x:c>
       <x:c r="C37" s="12" t="n">
@@ -4278,7 +4758,7 @@
       <x:c r="R37" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L37+N37))</x:f>
       </x:c>
-      <x:c r="S37" s="30" t="n">
+      <x:c r="S37" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A37</x:f>
         <x:v>0.8747195858336252</x:v>
       </x:c>
@@ -4298,12 +4778,27 @@
         <x:f>IF(Q37="","",Q37*S37)</x:f>
         <x:v>6.187306104233738</x:v>
       </x:c>
+      <x:c r="X37" s="12" t="n">
+        <x:f>IF(V37="","",X36+V37)</x:f>
+        <x:v>12.700064347257102</x:v>
+      </x:c>
+      <x:c r="Y37" s="12" t="n">
+        <x:f>IF(W37="","",Y36+W37)</x:f>
+        <x:v>-228.55381309019552</x:v>
+      </x:c>
+      <x:c r="Z37" s="30" t="n">
+        <x:f>IF(AND(X37&gt;=0,X36&lt;0),A37,"")</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="AA37" s="30" t="str">
+        <x:f>IF(AND(Y37&gt;=0,Y36&lt;0),A37,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="29" t="n">
+      <x:c r="A38" s="30" t="n">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B38" s="28" t="n">
+      <x:c r="B38" s="29" t="n">
         <x:v>46966</x:v>
       </x:c>
       <x:c r="C38" s="12" t="n">
@@ -4368,7 +4863,7 @@
       <x:c r="R38" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L38+N38))</x:f>
       </x:c>
-      <x:c r="S38" s="30" t="n">
+      <x:c r="S38" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A38</x:f>
         <x:v>0.8708255163153843</x:v>
       </x:c>
@@ -4388,12 +4883,26 @@
         <x:f>IF(Q38="","",Q38*S38)</x:f>
         <x:v>6.159761505380883</x:v>
       </x:c>
+      <x:c r="X38" s="12" t="n">
+        <x:f>IF(V38="","",X37+V38)</x:f>
+        <x:v>26.358678538733024</x:v>
+      </x:c>
+      <x:c r="Y38" s="12" t="n">
+        <x:f>IF(W38="","",Y37+W38)</x:f>
+        <x:v>-222.39405158481463</x:v>
+      </x:c>
+      <x:c r="Z38" s="30" t="str">
+        <x:f>IF(AND(X38&gt;=0,X37&lt;0),A38,"")</x:f>
+      </x:c>
+      <x:c r="AA38" s="30" t="str">
+        <x:f>IF(AND(Y38&gt;=0,Y37&lt;0),A38,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="29" t="n">
+      <x:c r="A39" s="30" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B39" s="28" t="n">
+      <x:c r="B39" s="29" t="n">
         <x:v>46997</x:v>
       </x:c>
       <x:c r="C39" s="12" t="n">
@@ -4458,7 +4967,7 @@
       <x:c r="R39" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L39+N39))</x:f>
       </x:c>
-      <x:c r="S39" s="30" t="n">
+      <x:c r="S39" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A39</x:f>
         <x:v>0.8669487823840657</x:v>
       </x:c>
@@ -4478,12 +4987,26 @@
         <x:f>IF(Q39="","",Q39*S39)</x:f>
         <x:v>6.132339529348555</x:v>
       </x:c>
+      <x:c r="X39" s="12" t="n">
+        <x:f>IF(V39="","",X38+V39)</x:f>
+        <x:v>39.95648742294725</x:v>
+      </x:c>
+      <x:c r="Y39" s="12" t="n">
+        <x:f>IF(W39="","",Y38+W39)</x:f>
+        <x:v>-216.2617120554661</x:v>
+      </x:c>
+      <x:c r="Z39" s="30" t="str">
+        <x:f>IF(AND(X39&gt;=0,X38&lt;0),A39,"")</x:f>
+      </x:c>
+      <x:c r="AA39" s="30" t="str">
+        <x:f>IF(AND(Y39&gt;=0,Y38&lt;0),A39,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="29" t="n">
+      <x:c r="A40" s="30" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B40" s="28" t="n">
+      <x:c r="B40" s="29" t="n">
         <x:v>47027</x:v>
       </x:c>
       <x:c r="C40" s="12" t="n">
@@ -4548,7 +5071,7 @@
       <x:c r="R40" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L40+N40))</x:f>
       </x:c>
-      <x:c r="S40" s="30" t="n">
+      <x:c r="S40" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A40</x:f>
         <x:v>0.863089306865245</x:v>
       </x:c>
@@ -4568,12 +5091,26 @@
         <x:f>IF(Q40="","",Q40*S40)</x:f>
         <x:v>6.105039630245482</x:v>
       </x:c>
+      <x:c r="X40" s="12" t="n">
+        <x:f>IF(V40="","",X39+V40)</x:f>
+        <x:v>53.49376169247073</x:v>
+      </x:c>
+      <x:c r="Y40" s="12" t="n">
+        <x:f>IF(W40="","",Y39+W40)</x:f>
+        <x:v>-210.15667242522062</x:v>
+      </x:c>
+      <x:c r="Z40" s="30" t="str">
+        <x:f>IF(AND(X40&gt;=0,X39&lt;0),A40,"")</x:f>
+      </x:c>
+      <x:c r="AA40" s="30" t="str">
+        <x:f>IF(AND(Y40&gt;=0,Y39&lt;0),A40,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="29" t="n">
+      <x:c r="A41" s="30" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="B41" s="28" t="n">
+      <x:c r="B41" s="29" t="n">
         <x:v>47058</x:v>
       </x:c>
       <x:c r="C41" s="12" t="n">
@@ -4638,7 +5175,7 @@
       <x:c r="R41" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L41+N41))</x:f>
       </x:c>
-      <x:c r="S41" s="30" t="n">
+      <x:c r="S41" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A41</x:f>
         <x:v>0.859247012928062</x:v>
       </x:c>
@@ -4658,12 +5195,26 @@
         <x:f>IF(Q41="","",Q41*S41)</x:f>
         <x:v>6.0778612646105845</x:v>
       </x:c>
+      <x:c r="X41" s="12" t="n">
+        <x:f>IF(V41="","",X40+V41)</x:f>
+        <x:v>66.97077083480744</x:v>
+      </x:c>
+      <x:c r="Y41" s="12" t="n">
+        <x:f>IF(W41="","",Y40+W41)</x:f>
+        <x:v>-204.07881116061003</x:v>
+      </x:c>
+      <x:c r="Z41" s="30" t="str">
+        <x:f>IF(AND(X41&gt;=0,X40&lt;0),A41,"")</x:f>
+      </x:c>
+      <x:c r="AA41" s="30" t="str">
+        <x:f>IF(AND(Y41&gt;=0,Y40&lt;0),A41,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="29" t="n">
+      <x:c r="A42" s="30" t="n">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="B42" s="28" t="n">
+      <x:c r="B42" s="29" t="n">
         <x:v>47088</x:v>
       </x:c>
       <x:c r="C42" s="12" t="n">
@@ -4728,7 +5279,7 @@
       <x:c r="R42" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L42+N42))</x:f>
       </x:c>
-      <x:c r="S42" s="30" t="n">
+      <x:c r="S42" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A42</x:f>
         <x:v>0.855421824083692</x:v>
       </x:c>
@@ -4748,12 +5299,26 @@
         <x:f>IF(Q42="","",Q42*S42)</x:f>
         <x:v>6.050803891402162</x:v>
       </x:c>
+      <x:c r="X42" s="12" t="n">
+        <x:f>IF(V42="","",X41+V42)</x:f>
+        <x:v>80.38778313775909</x:v>
+      </x:c>
+      <x:c r="Y42" s="12" t="n">
+        <x:f>IF(W42="","",Y41+W42)</x:f>
+        <x:v>-198.02800726920788</x:v>
+      </x:c>
+      <x:c r="Z42" s="30" t="str">
+        <x:f>IF(AND(X42&gt;=0,X41&lt;0),A42,"")</x:f>
+      </x:c>
+      <x:c r="AA42" s="30" t="str">
+        <x:f>IF(AND(Y42&gt;=0,Y41&lt;0),A42,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="29" t="n">
+      <x:c r="A43" s="30" t="n">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="B43" s="28" t="n">
+      <x:c r="B43" s="29" t="n">
         <x:v>47119</x:v>
       </x:c>
       <x:c r="C43" s="12" t="n">
@@ -4818,7 +5383,7 @@
       <x:c r="R43" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L43+N43))</x:f>
       </x:c>
-      <x:c r="S43" s="30" t="n">
+      <x:c r="S43" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A43</x:f>
         <x:v>0.8516136641838221</x:v>
       </x:c>
@@ -4838,12 +5403,26 @@
         <x:f>IF(Q43="","",Q43*S43)</x:f>
         <x:v>6.023866971987115</x:v>
       </x:c>
+      <x:c r="X43" s="12" t="n">
+        <x:f>IF(V43="","",X42+V43)</x:f>
+        <x:v>93.74506569476593</x:v>
+      </x:c>
+      <x:c r="Y43" s="12" t="n">
+        <x:f>IF(W43="","",Y42+W43)</x:f>
+        <x:v>-192.00414029722077</x:v>
+      </x:c>
+      <x:c r="Z43" s="30" t="str">
+        <x:f>IF(AND(X43&gt;=0,X42&lt;0),A43,"")</x:f>
+      </x:c>
+      <x:c r="AA43" s="30" t="str">
+        <x:f>IF(AND(Y43&gt;=0,Y42&lt;0),A43,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="29" t="n">
+      <x:c r="A44" s="30" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B44" s="28" t="n">
+      <x:c r="B44" s="29" t="n">
         <x:v>47150</x:v>
       </x:c>
       <x:c r="C44" s="12" t="n">
@@ -4908,7 +5487,7 @@
       <x:c r="R44" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L44+N44))</x:f>
       </x:c>
-      <x:c r="S44" s="30" t="n">
+      <x:c r="S44" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A44</x:f>
         <x:v>0.8478224574191363</x:v>
       </x:c>
@@ -4928,12 +5507,26 @@
         <x:f>IF(Q44="","",Q44*S44)</x:f>
         <x:v>5.997049970130232</x:v>
       </x:c>
+      <x:c r="X44" s="12" t="n">
+        <x:f>IF(V44="","",X43+V44)</x:f>
+        <x:v>107.04288441022382</x:v>
+      </x:c>
+      <x:c r="Y44" s="12" t="n">
+        <x:f>IF(W44="","",Y43+W44)</x:f>
+        <x:v>-186.00709032709054</x:v>
+      </x:c>
+      <x:c r="Z44" s="30" t="str">
+        <x:f>IF(AND(X44&gt;=0,X43&lt;0),A44,"")</x:f>
+      </x:c>
+      <x:c r="AA44" s="30" t="str">
+        <x:f>IF(AND(Y44&gt;=0,Y43&lt;0),A44,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="29" t="n">
+      <x:c r="A45" s="30" t="n">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="B45" s="28" t="n">
+      <x:c r="B45" s="29" t="n">
         <x:v>47178</x:v>
       </x:c>
       <x:c r="C45" s="12" t="n">
@@ -4998,7 +5591,7 @@
       <x:c r="R45" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L45+N45))</x:f>
       </x:c>
-      <x:c r="S45" s="30" t="n">
+      <x:c r="S45" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A45</x:f>
         <x:v>0.8440481283178054</x:v>
       </x:c>
@@ -5018,12 +5611,26 @@
         <x:f>IF(Q45="","",Q45*S45)</x:f>
         <x:v>5.970352351983502</x:v>
       </x:c>
+      <x:c r="X45" s="12" t="n">
+        <x:f>IF(V45="","",X44+V45)</x:f>
+        <x:v>120.2815040047776</x:v>
+      </x:c>
+      <x:c r="Y45" s="12" t="n">
+        <x:f>IF(W45="","",Y44+W45)</x:f>
+        <x:v>-180.03673797510703</x:v>
+      </x:c>
+      <x:c r="Z45" s="30" t="str">
+        <x:f>IF(AND(X45&gt;=0,X44&lt;0),A45,"")</x:f>
+      </x:c>
+      <x:c r="AA45" s="30" t="str">
+        <x:f>IF(AND(Y45&gt;=0,Y44&lt;0),A45,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="29" t="n">
+      <x:c r="A46" s="30" t="n">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B46" s="28" t="n">
+      <x:c r="B46" s="29" t="n">
         <x:v>47209</x:v>
       </x:c>
       <x:c r="C46" s="12" t="n">
@@ -5088,7 +5695,7 @@
       <x:c r="R46" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L46+N46))</x:f>
       </x:c>
-      <x:c r="S46" s="30" t="n">
+      <x:c r="S46" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A46</x:f>
         <x:v>0.8402906017439854</x:v>
       </x:c>
@@ -5108,12 +5715,26 @@
         <x:f>IF(Q46="","",Q46*S46)</x:f>
         <x:v>5.943773586075499</x:v>
       </x:c>
+      <x:c r="X46" s="12" t="n">
+        <x:f>IF(V46="","",X45+V46)</x:f>
+        <x:v>133.4611880205909</x:v>
+      </x:c>
+      <x:c r="Y46" s="12" t="n">
+        <x:f>IF(W46="","",Y45+W46)</x:f>
+        <x:v>-174.09296438903152</x:v>
+      </x:c>
+      <x:c r="Z46" s="30" t="str">
+        <x:f>IF(AND(X46&gt;=0,X45&lt;0),A46,"")</x:f>
+      </x:c>
+      <x:c r="AA46" s="30" t="str">
+        <x:f>IF(AND(Y46&gt;=0,Y45&lt;0),A46,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="29" t="n">
+      <x:c r="A47" s="30" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="B47" s="28" t="n">
+      <x:c r="B47" s="29" t="n">
         <x:v>47239</x:v>
       </x:c>
       <x:c r="C47" s="12" t="n">
@@ -5178,7 +5799,7 @@
       <x:c r="R47" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L47+N47))</x:f>
       </x:c>
-      <x:c r="S47" s="30" t="n">
+      <x:c r="S47" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A47</x:f>
         <x:v>0.8365498028963214</x:v>
       </x:c>
@@ -5198,12 +5819,26 @@
         <x:f>IF(Q47="","",Q47*S47)</x:f>
         <x:v>5.917313143300797</x:v>
       </x:c>
+      <x:c r="X47" s="12" t="n">
+        <x:f>IF(V47="","",X46+V47)</x:f>
+        <x:v>146.5821988265925</x:v>
+      </x:c>
+      <x:c r="Y47" s="12" t="n">
+        <x:f>IF(W47="","",Y46+W47)</x:f>
+        <x:v>-168.17565124573073</x:v>
+      </x:c>
+      <x:c r="Z47" s="30" t="str">
+        <x:f>IF(AND(X47&gt;=0,X46&lt;0),A47,"")</x:f>
+      </x:c>
+      <x:c r="AA47" s="30" t="str">
+        <x:f>IF(AND(Y47&gt;=0,Y46&lt;0),A47,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="29" t="n">
+      <x:c r="A48" s="30" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="B48" s="28" t="n">
+      <x:c r="B48" s="29" t="n">
         <x:v>47270</x:v>
       </x:c>
       <x:c r="C48" s="12" t="n">
@@ -5268,7 +5903,7 @@
       <x:c r="R48" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L48+N48))</x:f>
       </x:c>
-      <x:c r="S48" s="30" t="n">
+      <x:c r="S48" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A48</x:f>
         <x:v>0.8328256573064585</x:v>
       </x:c>
@@ -5288,12 +5923,26 @@
         <x:f>IF(Q48="","",Q48*S48)</x:f>
         <x:v>5.890970496909435</x:v>
       </x:c>
+      <x:c r="X48" s="12" t="n">
+        <x:f>IF(V48="","",X47+V48)</x:f>
+        <x:v>159.6447976236993</x:v>
+      </x:c>
+      <x:c r="Y48" s="12" t="n">
+        <x:f>IF(W48="","",Y47+W48)</x:f>
+        <x:v>-162.2846807488213</x:v>
+      </x:c>
+      <x:c r="Z48" s="30" t="str">
+        <x:f>IF(AND(X48&gt;=0,X47&lt;0),A48,"")</x:f>
+      </x:c>
+      <x:c r="AA48" s="30" t="str">
+        <x:f>IF(AND(Y48&gt;=0,Y47&lt;0),A48,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="29" t="n">
+      <x:c r="A49" s="30" t="n">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B49" s="28" t="n">
+      <x:c r="B49" s="29" t="n">
         <x:v>47300</x:v>
       </x:c>
       <x:c r="C49" s="12" t="n">
@@ -5358,7 +6007,7 @@
       <x:c r="R49" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L49+N49))</x:f>
       </x:c>
-      <x:c r="S49" s="30" t="n">
+      <x:c r="S49" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A49</x:f>
         <x:v>0.8291180908375594</x:v>
       </x:c>
@@ -5378,12 +6027,26 @@
         <x:f>IF(Q49="","",Q49*S49)</x:f>
         <x:v>5.8647451224964335</x:v>
       </x:c>
+      <x:c r="X49" s="12" t="n">
+        <x:f>IF(V49="","",X48+V49)</x:f>
+        <x:v>172.64924445001614</x:v>
+      </x:c>
+      <x:c r="Y49" s="12" t="n">
+        <x:f>IF(W49="","",Y48+W49)</x:f>
+        <x:v>-156.41993562632487</x:v>
+      </x:c>
+      <x:c r="Z49" s="30" t="str">
+        <x:f>IF(AND(X49&gt;=0,X48&lt;0),A49,"")</x:f>
+      </x:c>
+      <x:c r="AA49" s="30" t="str">
+        <x:f>IF(AND(Y49&gt;=0,Y48&lt;0),A49,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="29" t="n">
+      <x:c r="A50" s="30" t="n">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="B50" s="28" t="n">
+      <x:c r="B50" s="29" t="n">
         <x:v>47331</x:v>
       </x:c>
       <x:c r="C50" s="12" t="n">
@@ -5448,7 +6111,7 @@
       <x:c r="R50" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L50+N50))</x:f>
       </x:c>
-      <x:c r="S50" s="30" t="n">
+      <x:c r="S50" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A50</x:f>
         <x:v>0.8254270296828286</x:v>
       </x:c>
@@ -5468,12 +6131,26 @@
         <x:f>IF(Q50="","",Q50*S50)</x:f>
         <x:v>5.838636497991358</x:v>
       </x:c>
+      <x:c r="X50" s="12" t="n">
+        <x:f>IF(V50="","",X49+V50)</x:f>
+        <x:v>185.59579818601227</x:v>
+      </x:c>
+      <x:c r="Y50" s="12" t="n">
+        <x:f>IF(W50="","",Y49+W50)</x:f>
+        <x:v>-150.5812991283335</x:v>
+      </x:c>
+      <x:c r="Z50" s="30" t="str">
+        <x:f>IF(AND(X50&gt;=0,X49&lt;0),A50,"")</x:f>
+      </x:c>
+      <x:c r="AA50" s="30" t="str">
+        <x:f>IF(AND(Y50&gt;=0,Y49&lt;0),A50,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="29" t="n">
+      <x:c r="A51" s="30" t="n">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="B51" s="28" t="n">
+      <x:c r="B51" s="29" t="n">
         <x:v>47362</x:v>
       </x:c>
       <x:c r="C51" s="12" t="n">
@@ -5538,7 +6215,7 @@
       <x:c r="R51" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L51+N51))</x:f>
       </x:c>
-      <x:c r="S51" s="30" t="n">
+      <x:c r="S51" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A51</x:f>
         <x:v>0.8217524003640432</x:v>
       </x:c>
@@ -5558,12 +6235,26 @@
         <x:f>IF(Q51="","",Q51*S51)</x:f>
         <x:v>5.812644103647918</x:v>
       </x:c>
+      <x:c r="X51" s="12" t="n">
+        <x:f>IF(V51="","",X50+V51)</x:f>
+        <x:v>198.48471655967504</x:v>
+      </x:c>
+      <x:c r="Y51" s="12" t="n">
+        <x:f>IF(W51="","",Y50+W51)</x:f>
+        <x:v>-144.7686550246856</x:v>
+      </x:c>
+      <x:c r="Z51" s="30" t="str">
+        <x:f>IF(AND(X51&gt;=0,X50&lt;0),A51,"")</x:f>
+      </x:c>
+      <x:c r="AA51" s="30" t="str">
+        <x:f>IF(AND(Y51&gt;=0,Y50&lt;0),A51,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="29" t="n">
+      <x:c r="A52" s="30" t="n">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B52" s="28" t="n">
+      <x:c r="B52" s="29" t="n">
         <x:v>47392</x:v>
       </x:c>
       <x:c r="C52" s="12" t="n">
@@ -5628,7 +6319,7 @@
       <x:c r="R52" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L52+N52))</x:f>
       </x:c>
-      <x:c r="S52" s="30" t="n">
+      <x:c r="S52" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A52</x:f>
         <x:v>0.8180941297300899</x:v>
       </x:c>
@@ -5648,12 +6339,26 @@
         <x:f>IF(Q52="","",Q52*S52)</x:f>
         <x:v>5.786767422033631</x:v>
       </x:c>
+      <x:c r="X52" s="12" t="n">
+        <x:f>IF(V52="","",X51+V52)</x:f>
+        <x:v>211.3162561516404</x:v>
+      </x:c>
+      <x:c r="Y52" s="12" t="n">
+        <x:f>IF(W52="","",Y51+W52)</x:f>
+        <x:v>-138.98188760265197</x:v>
+      </x:c>
+      <x:c r="Z52" s="30" t="str">
+        <x:f>IF(AND(X52&gt;=0,X51&lt;0),A52,"")</x:f>
+      </x:c>
+      <x:c r="AA52" s="30" t="str">
+        <x:f>IF(AND(Y52&gt;=0,Y51&lt;0),A52,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="29" t="n">
+      <x:c r="A53" s="30" t="n">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="B53" s="28" t="n">
+      <x:c r="B53" s="29" t="n">
         <x:v>47423</x:v>
       </x:c>
       <x:c r="C53" s="12" t="n">
@@ -5718,7 +6423,7 @@
       <x:c r="R53" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L53+N53))</x:f>
       </x:c>
-      <x:c r="S53" s="30" t="n">
+      <x:c r="S53" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A53</x:f>
         <x:v>0.814452144955509</x:v>
       </x:c>
@@ -5738,12 +6443,26 @@
         <x:f>IF(Q53="","",Q53*S53)</x:f>
         <x:v>5.761005938019511</x:v>
       </x:c>
+      <x:c r="X53" s="12" t="n">
+        <x:f>IF(V53="","",X52+V53)</x:f>
+        <x:v>224.0906724003008</x:v>
+      </x:c>
+      <x:c r="Y53" s="12" t="n">
+        <x:f>IF(W53="","",Y52+W53)</x:f>
+        <x:v>-133.22088166463246</x:v>
+      </x:c>
+      <x:c r="Z53" s="30" t="str">
+        <x:f>IF(AND(X53&gt;=0,X52&lt;0),A53,"")</x:f>
+      </x:c>
+      <x:c r="AA53" s="30" t="str">
+        <x:f>IF(AND(Y53&gt;=0,Y52&lt;0),A53,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="29" t="n">
+      <x:c r="A54" s="30" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B54" s="28" t="n">
+      <x:c r="B54" s="29" t="n">
         <x:v>47453</x:v>
       </x:c>
       <x:c r="C54" s="12" t="n">
@@ -5808,7 +6527,7 @@
       <x:c r="R54" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L54+N54))</x:f>
       </x:c>
-      <x:c r="S54" s="30" t="n">
+      <x:c r="S54" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A54</x:f>
         <x:v>0.8108263735390445</x:v>
       </x:c>
@@ -5828,12 +6547,26 @@
         <x:f>IF(Q54="","",Q54*S54)</x:f>
         <x:v>5.735359138769821</x:v>
       </x:c>
+      <x:c r="X54" s="12" t="n">
+        <x:f>IF(V54="","",X53+V54)</x:f>
+        <x:v>236.80821960689005</x:v>
+      </x:c>
+      <x:c r="Y54" s="12" t="n">
+        <x:f>IF(W54="","",Y53+W54)</x:f>
+        <x:v>-127.48552252586263</x:v>
+      </x:c>
+      <x:c r="Z54" s="30" t="str">
+        <x:f>IF(AND(X54&gt;=0,X53&lt;0),A54,"")</x:f>
+      </x:c>
+      <x:c r="AA54" s="30" t="str">
+        <x:f>IF(AND(Y54&gt;=0,Y53&lt;0),A54,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="29" t="n">
+      <x:c r="A55" s="30" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="B55" s="28" t="n">
+      <x:c r="B55" s="29" t="n">
         <x:v>47484</x:v>
       </x:c>
       <x:c r="C55" s="12" t="n">
@@ -5898,7 +6631,7 @@
       <x:c r="R55" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L55+N55))</x:f>
       </x:c>
-      <x:c r="S55" s="30" t="n">
+      <x:c r="S55" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A55</x:f>
         <x:v>0.8072167433022012</x:v>
       </x:c>
@@ -5918,12 +6651,26 @@
         <x:f>IF(Q55="","",Q55*S55)</x:f>
         <x:v>5.709826513731864</x:v>
       </x:c>
+      <x:c r="X55" s="12" t="n">
+        <x:f>IF(V55="","",X54+V55)</x:f>
+        <x:v>249.46915094054583</x:v>
+      </x:c>
+      <x:c r="Y55" s="12" t="n">
+        <x:f>IF(W55="","",Y54+W55)</x:f>
+        <x:v>-121.77569601213077</x:v>
+      </x:c>
+      <x:c r="Z55" s="30" t="str">
+        <x:f>IF(AND(X55&gt;=0,X54&lt;0),A55,"")</x:f>
+      </x:c>
+      <x:c r="AA55" s="30" t="str">
+        <x:f>IF(AND(Y55&gt;=0,Y54&lt;0),A55,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="29" t="n">
+      <x:c r="A56" s="30" t="n">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="B56" s="28" t="n">
+      <x:c r="B56" s="29" t="n">
         <x:v>47515</x:v>
       </x:c>
       <x:c r="C56" s="12" t="n">
@@ -5988,7 +6735,7 @@
       <x:c r="R56" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L56+N56))</x:f>
       </x:c>
-      <x:c r="S56" s="30" t="n">
+      <x:c r="S56" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A56</x:f>
         <x:v>0.8036231823878068</x:v>
       </x:c>
@@ -6008,12 +6755,26 @@
         <x:f>IF(Q56="","",Q56*S56)</x:f>
         <x:v>5.684407554625811</x:v>
       </x:c>
+      <x:c r="X56" s="12" t="n">
+        <x:f>IF(V56="","",X55+V56)</x:f>
+        <x:v>262.07371844334955</x:v>
+      </x:c>
+      <x:c r="Y56" s="12" t="n">
+        <x:f>IF(W56="","",Y55+W56)</x:f>
+        <x:v>-116.09128845750496</x:v>
+      </x:c>
+      <x:c r="Z56" s="30" t="str">
+        <x:f>IF(AND(X56&gt;=0,X55&lt;0),A56,"")</x:f>
+      </x:c>
+      <x:c r="AA56" s="30" t="str">
+        <x:f>IF(AND(Y56&gt;=0,Y55&lt;0),A56,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="29" t="n">
+      <x:c r="A57" s="30" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="B57" s="28" t="n">
+      <x:c r="B57" s="29" t="n">
         <x:v>47543</x:v>
       </x:c>
       <x:c r="C57" s="12" t="n">
@@ -6078,7 +6839,7 @@
       <x:c r="R57" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L57+N57))</x:f>
       </x:c>
-      <x:c r="S57" s="30" t="n">
+      <x:c r="S57" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A57</x:f>
         <x:v>0.8000456192585832</x:v>
       </x:c>
@@ -6098,12 +6859,26 @@
         <x:f>IF(Q57="","",Q57*S57)</x:f>
         <x:v>5.659101755434598</x:v>
       </x:c>
+      <x:c r="X57" s="12" t="n">
+        <x:f>IF(V57="","",X56+V57)</x:f>
+        <x:v>274.6221730353437</x:v>
+      </x:c>
+      <x:c r="Y57" s="12" t="n">
+        <x:f>IF(W57="","",Y56+W57)</x:f>
+        <x:v>-110.43218670207037</x:v>
+      </x:c>
+      <x:c r="Z57" s="30" t="str">
+        <x:f>IF(AND(X57&gt;=0,X56&lt;0),A57,"")</x:f>
+      </x:c>
+      <x:c r="AA57" s="30" t="str">
+        <x:f>IF(AND(Y57&gt;=0,Y56&lt;0),A57,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="29" t="n">
+      <x:c r="A58" s="30" t="n">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B58" s="28" t="n">
+      <x:c r="B58" s="29" t="n">
         <x:v>47574</x:v>
       </x:c>
       <x:c r="C58" s="12" t="n">
@@ -6168,7 +6943,7 @@
       <x:c r="R58" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L58+N58))</x:f>
       </x:c>
-      <x:c r="S58" s="30" t="n">
+      <x:c r="S58" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A58</x:f>
         <x:v>0.7964839826957206</x:v>
       </x:c>
@@ -6188,12 +6963,26 @@
         <x:f>IF(Q58="","",Q58*S58)</x:f>
         <x:v>5.633908612393837</x:v>
       </x:c>
+      <x:c r="X58" s="12" t="n">
+        <x:f>IF(V58="","",X57+V58)</x:f>
+        <x:v>287.1147645195269</x:v>
+      </x:c>
+      <x:c r="Y58" s="12" t="n">
+        <x:f>IF(W58="","",Y57+W58)</x:f>
+        <x:v>-104.79827808967653</x:v>
+      </x:c>
+      <x:c r="Z58" s="30" t="str">
+        <x:f>IF(AND(X58&gt;=0,X57&lt;0),A58,"")</x:f>
+      </x:c>
+      <x:c r="AA58" s="30" t="str">
+        <x:f>IF(AND(Y58&gt;=0,Y57&lt;0),A58,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="29" t="n">
+      <x:c r="A59" s="30" t="n">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="B59" s="28" t="n">
+      <x:c r="B59" s="29" t="n">
         <x:v>47604</x:v>
       </x:c>
       <x:c r="C59" s="12" t="n">
@@ -6258,7 +7047,7 @@
       <x:c r="R59" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L59+N59))</x:f>
       </x:c>
-      <x:c r="S59" s="30" t="n">
+      <x:c r="S59" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A59</x:f>
         <x:v>0.792938201797461</x:v>
       </x:c>
@@ -6278,12 +7067,26 @@
         <x:f>IF(Q59="","",Q59*S59)</x:f>
         <x:v>5.608827623981798</x:v>
       </x:c>
+      <x:c r="X59" s="12" t="n">
+        <x:f>IF(V59="","",X58+V59)</x:f>
+        <x:v>299.551741586827</x:v>
+      </x:c>
+      <x:c r="Y59" s="12" t="n">
+        <x:f>IF(W59="","",Y58+W59)</x:f>
+        <x:v>-99.18945046569473</x:v>
+      </x:c>
+      <x:c r="Z59" s="30" t="str">
+        <x:f>IF(AND(X59&gt;=0,X58&lt;0),A59,"")</x:f>
+      </x:c>
+      <x:c r="AA59" s="30" t="str">
+        <x:f>IF(AND(Y59&gt;=0,Y58&lt;0),A59,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="60">
-      <x:c r="A60" s="29" t="n">
+      <x:c r="A60" s="30" t="n">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="B60" s="28" t="n">
+      <x:c r="B60" s="29" t="n">
         <x:v>47635</x:v>
       </x:c>
       <x:c r="C60" s="12" t="n">
@@ -6348,7 +7151,7 @@
       <x:c r="R60" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L60+N60))</x:f>
       </x:c>
-      <x:c r="S60" s="30" t="n">
+      <x:c r="S60" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A60</x:f>
         <x:v>0.7894082059776857</x:v>
       </x:c>
@@ -6368,12 +7171,26 @@
         <x:f>IF(Q60="","",Q60*S60)</x:f>
         <x:v>5.583858290909416</x:v>
       </x:c>
+      <x:c r="X60" s="12" t="n">
+        <x:f>IF(V60="","",X59+V60)</x:f>
+        <x:v>311.9333518210515</x:v>
+      </x:c>
+      <x:c r="Y60" s="12" t="n">
+        <x:f>IF(W60="","",Y59+W60)</x:f>
+        <x:v>-93.60559217478531</x:v>
+      </x:c>
+      <x:c r="Z60" s="30" t="str">
+        <x:f>IF(AND(X60&gt;=0,X59&lt;0),A60,"")</x:f>
+      </x:c>
+      <x:c r="AA60" s="30" t="str">
+        <x:f>IF(AND(Y60&gt;=0,Y59&lt;0),A60,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="61">
-      <x:c r="A61" s="29" t="n">
+      <x:c r="A61" s="30" t="n">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="B61" s="28" t="n">
+      <x:c r="B61" s="29" t="n">
         <x:v>47665</x:v>
       </x:c>
       <x:c r="C61" s="12" t="n">
@@ -6438,7 +7255,7 @@
       <x:c r="R61" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L61+N61))</x:f>
       </x:c>
-      <x:c r="S61" s="30" t="n">
+      <x:c r="S61" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A61</x:f>
         <x:v>0.7858939249645112</x:v>
       </x:c>
@@ -6458,12 +7275,26 @@
         <x:f>IF(Q61="","",Q61*S61)</x:f>
         <x:v>5.559000116110363</x:v>
       </x:c>
+      <x:c r="X61" s="12" t="n">
+        <x:f>IF(V61="","",X60+V61)</x:f>
+        <x:v>324.2598417038162</x:v>
+      </x:c>
+      <x:c r="Y61" s="12" t="n">
+        <x:f>IF(W61="","",Y60+W61)</x:f>
+        <x:v>-88.04659205867495</x:v>
+      </x:c>
+      <x:c r="Z61" s="30" t="str">
+        <x:f>IF(AND(X61&gt;=0,X60&lt;0),A61,"")</x:f>
+      </x:c>
+      <x:c r="AA61" s="30" t="str">
+        <x:f>IF(AND(Y61&gt;=0,Y60&lt;0),A61,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="62">
-      <x:c r="A62" s="29" t="n">
+      <x:c r="A62" s="30" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="B62" s="28" t="n">
+      <x:c r="B62" s="29" t="n">
         <x:v>47696</x:v>
       </x:c>
       <x:c r="C62" s="12" t="n">
@@ -6528,7 +7359,7 @@
       <x:c r="R62" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L62+N62))</x:f>
       </x:c>
-      <x:c r="S62" s="30" t="n">
+      <x:c r="S62" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A62</x:f>
         <x:v>0.7823952887988896</x:v>
       </x:c>
@@ -6548,12 +7379,26 @@
         <x:f>IF(Q62="","",Q62*S62)</x:f>
         <x:v>5.534252604731145</x:v>
       </x:c>
+      <x:c r="X62" s="12" t="n">
+        <x:f>IF(V62="","",X61+V62)</x:f>
+        <x:v>336.53145661945234</x:v>
+      </x:c>
+      <x:c r="Y62" s="12" t="n">
+        <x:f>IF(W62="","",Y61+W62)</x:f>
+        <x:v>-82.5123394539438</x:v>
+      </x:c>
+      <x:c r="Z62" s="30" t="str">
+        <x:f>IF(AND(X62&gt;=0,X61&lt;0),A62,"")</x:f>
+      </x:c>
+      <x:c r="AA62" s="30" t="str">
+        <x:f>IF(AND(Y62&gt;=0,Y61&lt;0),A62,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="29" t="n">
+      <x:c r="A63" s="30" t="n">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="B63" s="28" t="n">
+      <x:c r="B63" s="29" t="n">
         <x:v>47727</x:v>
       </x:c>
       <x:c r="C63" s="12" t="n">
@@ -6618,7 +7463,7 @@
       <x:c r="R63" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L63+N63))</x:f>
       </x:c>
-      <x:c r="S63" s="30" t="n">
+      <x:c r="S63" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A63</x:f>
         <x:v>0.7789122278332162</x:v>
       </x:c>
@@ -6638,12 +7483,26 @@
         <x:f>IF(Q63="","",Q63*S63)</x:f>
         <x:v>5.5096152641212495</x:v>
       </x:c>
+      <x:c r="X63" s="12" t="n">
+        <x:f>IF(V63="","",X62+V63)</x:f>
+        <x:v>348.748440859891</x:v>
+      </x:c>
+      <x:c r="Y63" s="12" t="n">
+        <x:f>IF(W63="","",Y62+W63)</x:f>
+        <x:v>-77.00272418982254</x:v>
+      </x:c>
+      <x:c r="Z63" s="30" t="str">
+        <x:f>IF(AND(X63&gt;=0,X62&lt;0),A63,"")</x:f>
+      </x:c>
+      <x:c r="AA63" s="30" t="str">
+        <x:f>IF(AND(Y63&gt;=0,Y62&lt;0),A63,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="29" t="n">
+      <x:c r="A64" s="30" t="n">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="B64" s="28" t="n">
+      <x:c r="B64" s="29" t="n">
         <x:v>47757</x:v>
       </x:c>
       <x:c r="C64" s="12" t="n">
@@ -6708,7 +7567,7 @@
       <x:c r="R64" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L64+N64))</x:f>
       </x:c>
-      <x:c r="S64" s="30" t="n">
+      <x:c r="S64" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A64</x:f>
         <x:v>0.775444672729943</x:v>
       </x:c>
@@ -6728,12 +7587,26 @@
         <x:f>IF(Q64="","",Q64*S64)</x:f>
         <x:v>5.485087603823347</x:v>
       </x:c>
+      <x:c r="X64" s="12" t="n">
+        <x:f>IF(V64="","",X63+V64)</x:f>
+        <x:v>360.91103762952645</x:v>
+      </x:c>
+      <x:c r="Y64" s="12" t="n">
+        <x:f>IF(W64="","",Y63+W64)</x:f>
+        <x:v>-71.5176365859992</x:v>
+      </x:c>
+      <x:c r="Z64" s="30" t="str">
+        <x:f>IF(AND(X64&gt;=0,X63&lt;0),A64,"")</x:f>
+      </x:c>
+      <x:c r="AA64" s="30" t="str">
+        <x:f>IF(AND(Y64&gt;=0,Y63&lt;0),A64,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="65">
-      <x:c r="A65" s="29" t="n">
+      <x:c r="A65" s="30" t="n">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="B65" s="28" t="n">
+      <x:c r="B65" s="29" t="n">
         <x:v>47788</x:v>
       </x:c>
       <x:c r="C65" s="12" t="n">
@@ -6798,7 +7671,7 @@
       <x:c r="R65" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L65+N65))</x:f>
       </x:c>
-      <x:c r="S65" s="30" t="n">
+      <x:c r="S65" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A65</x:f>
         <x:v>0.7719925544601981</x:v>
       </x:c>
@@ -6818,12 +7691,26 @@
         <x:f>IF(Q65="","",Q65*S65)</x:f>
         <x:v>5.460669135563517</x:v>
       </x:c>
+      <x:c r="X65" s="12" t="n">
+        <x:f>IF(V65="","",X64+V65)</x:f>
+        <x:v>373.01948905005764</x:v>
+      </x:c>
+      <x:c r="Y65" s="12" t="n">
+        <x:f>IF(W65="","",Y64+W65)</x:f>
+        <x:v>-66.05696745043568</x:v>
+      </x:c>
+      <x:c r="Z65" s="30" t="str">
+        <x:f>IF(AND(X65&gt;=0,X64&lt;0),A65,"")</x:f>
+      </x:c>
+      <x:c r="AA65" s="30" t="str">
+        <x:f>IF(AND(Y65&gt;=0,Y64&lt;0),A65,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="66">
-      <x:c r="A66" s="29" t="n">
+      <x:c r="A66" s="30" t="n">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="B66" s="28" t="n">
+      <x:c r="B66" s="29" t="n">
         <x:v>47818</x:v>
       </x:c>
       <x:c r="C66" s="12" t="n">
@@ -6888,7 +7775,7 @@
       <x:c r="R66" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L66+N66))</x:f>
       </x:c>
-      <x:c r="S66" s="30" t="n">
+      <x:c r="S66" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A66</x:f>
         <x:v>0.7685558043024118</x:v>
       </x:c>
@@ -6908,12 +7795,26 @@
         <x:f>IF(Q66="","",Q66*S66)</x:f>
         <x:v>5.436359373241536</x:v>
       </x:c>
+      <x:c r="X66" s="12" t="n">
+        <x:f>IF(V66="","",X65+V66)</x:f>
+        <x:v>385.0740361653081</x:v>
+      </x:c>
+      <x:c r="Y66" s="12" t="n">
+        <x:f>IF(W66="","",Y65+W66)</x:f>
+        <x:v>-60.62060807719414</x:v>
+      </x:c>
+      <x:c r="Z66" s="30" t="str">
+        <x:f>IF(AND(X66&gt;=0,X65&lt;0),A66,"")</x:f>
+      </x:c>
+      <x:c r="AA66" s="30" t="str">
+        <x:f>IF(AND(Y66&gt;=0,Y65&lt;0),A66,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="67">
-      <x:c r="A67" s="29" t="n">
+      <x:c r="A67" s="30" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="B67" s="28" t="n">
+      <x:c r="B67" s="29" t="n">
         <x:v>47849</x:v>
       </x:c>
       <x:c r="C67" s="12" t="n">
@@ -6978,7 +7879,7 @@
       <x:c r="R67" s="12" t="str">
         <x:f>IF(OR(Supuestos!$B$12="",Supuestos!$B$13="",Supuestos!$B$14="",Supuestos!$B$16=""),"",-(L67+N67))</x:f>
       </x:c>
-      <x:c r="S67" s="30" t="n">
+      <x:c r="S67" s="31" t="n">
         <x:f>1/(1+Supuestos!$B$9)^A67</x:f>
         <x:v>0.7651343538409489</x:v>
       </x:c>
@@ -6998,11 +7899,25 @@
         <x:f>IF(Q67="","",Q67*S67)</x:f>
         <x:v>5.412157832921197</x:v>
       </x:c>
+      <x:c r="X67" s="12" t="n">
+        <x:f>IF(V67="","",X66+V67)</x:f>
+        <x:v>397.07491894602447</x:v>
+      </x:c>
+      <x:c r="Y67" s="12" t="n">
+        <x:f>IF(W67="","",Y66+W67)</x:f>
+        <x:v>-55.208450244272946</x:v>
+      </x:c>
+      <x:c r="Z67" s="30" t="str">
+        <x:f>IF(AND(X67&gt;=0,X66&lt;0),A67,"")</x:f>
+      </x:c>
+      <x:c r="AA67" s="30" t="str">
+        <x:f>IF(AND(Y67&gt;=0,Y66&lt;0),A67,"")</x:f>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:W1"/>
-    <x:mergeCell ref="A3:W3"/>
+    <x:mergeCell ref="A1:AA1"/>
+    <x:mergeCell ref="A3:AA3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7025,86 +7940,86 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="43" t="str">
+      <x:c r="A1" s="44" t="str">
         <x:v>FP-187 — Escenarios financieros</x:v>
       </x:c>
-      <x:c r="B1" s="43"/>
-      <x:c r="C1" s="43"/>
-      <x:c r="D1" s="43"/>
-      <x:c r="E1" s="43"/>
-      <x:c r="F1" s="43"/>
-      <x:c r="G1" s="43"/>
-      <x:c r="H1" s="43"/>
-      <x:c r="I1" s="43"/>
-      <x:c r="J1" s="43"/>
+      <x:c r="B1" s="44"/>
+      <x:c r="C1" s="44"/>
+      <x:c r="D1" s="44"/>
+      <x:c r="E1" s="44"/>
+      <x:c r="F1" s="44"/>
+      <x:c r="G1" s="44"/>
+      <x:c r="H1" s="44"/>
+      <x:c r="I1" s="44"/>
+      <x:c r="J1" s="44"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="44"/>
-      <x:c r="B2" s="44"/>
-      <x:c r="C2" s="44"/>
-      <x:c r="D2" s="44"/>
-      <x:c r="E2" s="44"/>
-      <x:c r="F2" s="44"/>
-      <x:c r="G2" s="44"/>
-      <x:c r="H2" s="44"/>
-      <x:c r="I2" s="44"/>
-      <x:c r="J2" s="44"/>
+      <x:c r="A2" s="45"/>
+      <x:c r="B2" s="45"/>
+      <x:c r="C2" s="45"/>
+      <x:c r="D2" s="45"/>
+      <x:c r="E2" s="45"/>
+      <x:c r="F2" s="45"/>
+      <x:c r="G2" s="45"/>
+      <x:c r="H2" s="45"/>
+      <x:c r="I2" s="45"/>
+      <x:c r="J2" s="45"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="44" t="str">
+      <x:c r="A3" s="45" t="str">
         <x:v>Esta vista separa el gasto cloud comparable del flujo incremental de optimización. Los valores de operación e implementación permanecen parametrizados.</x:v>
       </x:c>
-      <x:c r="B3" s="44"/>
-      <x:c r="C3" s="44"/>
-      <x:c r="D3" s="44"/>
-      <x:c r="E3" s="44"/>
-      <x:c r="F3" s="44"/>
-      <x:c r="G3" s="44"/>
-      <x:c r="H3" s="44"/>
-      <x:c r="I3" s="44"/>
-      <x:c r="J3" s="44"/>
+      <x:c r="B3" s="45"/>
+      <x:c r="C3" s="45"/>
+      <x:c r="D3" s="45"/>
+      <x:c r="E3" s="45"/>
+      <x:c r="F3" s="45"/>
+      <x:c r="G3" s="45"/>
+      <x:c r="H3" s="45"/>
+      <x:c r="I3" s="45"/>
+      <x:c r="J3" s="45"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="44"/>
-      <x:c r="B4" s="44"/>
-      <x:c r="C4" s="44"/>
-      <x:c r="D4" s="44"/>
-      <x:c r="E4" s="44"/>
-      <x:c r="F4" s="44"/>
-      <x:c r="G4" s="44"/>
-      <x:c r="H4" s="44"/>
-      <x:c r="I4" s="44"/>
-      <x:c r="J4" s="44"/>
+      <x:c r="A4" s="45"/>
+      <x:c r="B4" s="45"/>
+      <x:c r="C4" s="45"/>
+      <x:c r="D4" s="45"/>
+      <x:c r="E4" s="45"/>
+      <x:c r="F4" s="45"/>
+      <x:c r="G4" s="45"/>
+      <x:c r="H4" s="45"/>
+      <x:c r="I4" s="45"/>
+      <x:c r="J4" s="45"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="36" t="str">
+      <x:c r="A5" s="37" t="str">
         <x:v>Región</x:v>
       </x:c>
-      <x:c r="B5" s="36" t="str">
+      <x:c r="B5" s="37" t="str">
         <x:v>Escenario</x:v>
       </x:c>
-      <x:c r="C5" s="36" t="str">
+      <x:c r="C5" s="37" t="str">
         <x:v>Cloud 60m</x:v>
       </x:c>
-      <x:c r="D5" s="36" t="str">
+      <x:c r="D5" s="37" t="str">
         <x:v>Ahorro bruto 60m</x:v>
       </x:c>
-      <x:c r="E5" s="36" t="str">
+      <x:c r="E5" s="37" t="str">
         <x:v>Operación 60m</x:v>
       </x:c>
-      <x:c r="F5" s="36" t="str">
+      <x:c r="F5" s="37" t="str">
         <x:v>Implementación</x:v>
       </x:c>
-      <x:c r="G5" s="36" t="str">
+      <x:c r="G5" s="37" t="str">
         <x:v>VAN bruto</x:v>
       </x:c>
-      <x:c r="H5" s="36" t="str">
+      <x:c r="H5" s="37" t="str">
         <x:v>VAN incremental</x:v>
       </x:c>
-      <x:c r="I5" s="36" t="str">
+      <x:c r="I5" s="37" t="str">
         <x:v>TIR anual</x:v>
       </x:c>
-      <x:c r="J5" s="36" t="str">
+      <x:c r="J5" s="37" t="str">
         <x:v>Estado</x:v>
       </x:c>
     </x:row>
@@ -7141,9 +8056,9 @@
       <x:c r="I6" s="13" t="str">
         <x:f>""</x:f>
       </x:c>
-      <x:c r="J6" s="14" t="str">
+      <x:c r="J6" s="15" t="n">
         <x:f>'Resumen'!K5</x:f>
-        <x:v>Provisional: proxies públicos</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -7180,9 +8095,9 @@
         <x:f>'Resumen'!J5</x:f>
         <x:v>0.4391345109616156</x:v>
       </x:c>
-      <x:c r="J7" s="14" t="str">
+      <x:c r="J7" s="15" t="n">
         <x:f>'Resumen'!K5</x:f>
-        <x:v>Provisional: proxies públicos</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -7218,9 +8133,9 @@
       <x:c r="I8" s="13" t="str">
         <x:f>""</x:f>
       </x:c>
-      <x:c r="J8" s="14" t="str">
+      <x:c r="J8" s="15" t="str">
         <x:f>'Resumen'!K6</x:f>
-        <x:v>Provisional: proxies públicos</x:v>
+        <x:v>No recupera en 60 meses</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -7257,9 +8172,9 @@
         <x:f>'Resumen'!J6</x:f>
         <x:v>-0.002138745694702626</x:v>
       </x:c>
-      <x:c r="J9" s="14" t="str">
+      <x:c r="J9" s="15" t="str">
         <x:f>'Resumen'!K6</x:f>
-        <x:v>Provisional: proxies públicos</x:v>
+        <x:v>No recupera en 60 meses</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7286,72 +8201,72 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="43" t="str">
+      <x:c r="A1" s="44" t="str">
         <x:v>FP-187 — Fuentes y datos importados</x:v>
       </x:c>
-      <x:c r="B1" s="43"/>
-      <x:c r="C1" s="43"/>
-      <x:c r="D1" s="43"/>
-      <x:c r="E1" s="43"/>
-      <x:c r="F1" s="43"/>
-      <x:c r="G1" s="43"/>
-      <x:c r="H1" s="43"/>
+      <x:c r="B1" s="44"/>
+      <x:c r="C1" s="44"/>
+      <x:c r="D1" s="44"/>
+      <x:c r="E1" s="44"/>
+      <x:c r="F1" s="44"/>
+      <x:c r="G1" s="44"/>
+      <x:c r="H1" s="44"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="44"/>
-      <x:c r="B2" s="44"/>
-      <x:c r="C2" s="44"/>
-      <x:c r="D2" s="44"/>
-      <x:c r="E2" s="44"/>
-      <x:c r="F2" s="44"/>
-      <x:c r="G2" s="44"/>
-      <x:c r="H2" s="44"/>
+      <x:c r="A2" s="45"/>
+      <x:c r="B2" s="45"/>
+      <x:c r="C2" s="45"/>
+      <x:c r="D2" s="45"/>
+      <x:c r="E2" s="45"/>
+      <x:c r="F2" s="45"/>
+      <x:c r="G2" s="45"/>
+      <x:c r="H2" s="45"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="44" t="str">
+      <x:c r="A3" s="45" t="str">
         <x:v>Los costos base son un snapshot de FP-183; los ahorros son un snapshot de FP-184. Cambios futuros deben actualizar estos insumos y su trazabilidad.</x:v>
       </x:c>
-      <x:c r="B3" s="44"/>
-      <x:c r="C3" s="44"/>
-      <x:c r="D3" s="44"/>
-      <x:c r="E3" s="44"/>
-      <x:c r="F3" s="44"/>
-      <x:c r="G3" s="44"/>
-      <x:c r="H3" s="44"/>
+      <x:c r="B3" s="45"/>
+      <x:c r="C3" s="45"/>
+      <x:c r="D3" s="45"/>
+      <x:c r="E3" s="45"/>
+      <x:c r="F3" s="45"/>
+      <x:c r="G3" s="45"/>
+      <x:c r="H3" s="45"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="44"/>
-      <x:c r="B4" s="44"/>
-      <x:c r="C4" s="44"/>
-      <x:c r="D4" s="44"/>
-      <x:c r="E4" s="44"/>
-      <x:c r="F4" s="44"/>
-      <x:c r="G4" s="44"/>
-      <x:c r="H4" s="44"/>
+      <x:c r="A4" s="45"/>
+      <x:c r="B4" s="45"/>
+      <x:c r="C4" s="45"/>
+      <x:c r="D4" s="45"/>
+      <x:c r="E4" s="45"/>
+      <x:c r="F4" s="45"/>
+      <x:c r="G4" s="45"/>
+      <x:c r="H4" s="45"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="36" t="str">
+      <x:c r="A5" s="37" t="str">
         <x:v>Mes</x:v>
       </x:c>
-      <x:c r="B5" s="36" t="str">
+      <x:c r="B5" s="37" t="str">
         <x:v>Fecha</x:v>
       </x:c>
-      <x:c r="C5" s="36" t="str">
+      <x:c r="C5" s="37" t="str">
         <x:v>Chile Central base cloud</x:v>
       </x:c>
-      <x:c r="D5" s="36" t="str">
+      <x:c r="D5" s="37" t="str">
         <x:v>East US base cloud</x:v>
       </x:c>
-      <x:c r="E5" s="36" t="str">
+      <x:c r="E5" s="37" t="str">
         <x:v>Ahorro bruto Chile</x:v>
       </x:c>
-      <x:c r="F5" s="36" t="str">
+      <x:c r="F5" s="37" t="str">
         <x:v>Ahorro bruto East US</x:v>
       </x:c>
-      <x:c r="G5" s="36" t="str">
+      <x:c r="G5" s="37" t="str">
         <x:v>Fuente base</x:v>
       </x:c>
-      <x:c r="H5" s="36" t="str">
+      <x:c r="H5" s="37" t="str">
         <x:v>Fuente ahorro</x:v>
       </x:c>
     </x:row>
@@ -7359,7 +8274,7 @@
       <x:c r="A6" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B6" s="28" t="n">
+      <x:c r="B6" s="29" t="n">
         <x:v>46023</x:v>
       </x:c>
       <x:c r="C6" s="12" t="n">
@@ -7385,7 +8300,7 @@
       <x:c r="A7" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B7" s="28" t="n">
+      <x:c r="B7" s="29" t="n">
         <x:v>46054</x:v>
       </x:c>
       <x:c r="C7" s="12" t="n">
@@ -7411,7 +8326,7 @@
       <x:c r="A8" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B8" s="28" t="n">
+      <x:c r="B8" s="29" t="n">
         <x:v>46082</x:v>
       </x:c>
       <x:c r="C8" s="12" t="n">
@@ -7437,7 +8352,7 @@
       <x:c r="A9" s="11" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="n">
+      <x:c r="B9" s="29" t="n">
         <x:v>46113</x:v>
       </x:c>
       <x:c r="C9" s="12" t="n">
@@ -7463,7 +8378,7 @@
       <x:c r="A10" s="11" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="n">
+      <x:c r="B10" s="29" t="n">
         <x:v>46143</x:v>
       </x:c>
       <x:c r="C10" s="12" t="n">
@@ -7489,7 +8404,7 @@
       <x:c r="A11" s="11" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
+      <x:c r="B11" s="29" t="n">
         <x:v>46174</x:v>
       </x:c>
       <x:c r="C11" s="12" t="n">
@@ -7515,7 +8430,7 @@
       <x:c r="A12" s="11" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B12" s="28" t="n">
+      <x:c r="B12" s="29" t="n">
         <x:v>46204</x:v>
       </x:c>
       <x:c r="C12" s="12" t="n">
@@ -7541,7 +8456,7 @@
       <x:c r="A13" s="11" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B13" s="28" t="n">
+      <x:c r="B13" s="29" t="n">
         <x:v>46235</x:v>
       </x:c>
       <x:c r="C13" s="12" t="n">
@@ -7567,7 +8482,7 @@
       <x:c r="A14" s="11" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B14" s="28" t="n">
+      <x:c r="B14" s="29" t="n">
         <x:v>46266</x:v>
       </x:c>
       <x:c r="C14" s="12" t="n">
@@ -7593,7 +8508,7 @@
       <x:c r="A15" s="11" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B15" s="28" t="n">
+      <x:c r="B15" s="29" t="n">
         <x:v>46296</x:v>
       </x:c>
       <x:c r="C15" s="12" t="n">
@@ -7619,7 +8534,7 @@
       <x:c r="A16" s="11" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
+      <x:c r="B16" s="29" t="n">
         <x:v>46327</x:v>
       </x:c>
       <x:c r="C16" s="12" t="n">
@@ -7645,7 +8560,7 @@
       <x:c r="A17" s="11" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B17" s="28" t="n">
+      <x:c r="B17" s="29" t="n">
         <x:v>46357</x:v>
       </x:c>
       <x:c r="C17" s="12" t="n">
@@ -7671,7 +8586,7 @@
       <x:c r="A18" s="11" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B18" s="28" t="n">
+      <x:c r="B18" s="29" t="n">
         <x:v>46388</x:v>
       </x:c>
       <x:c r="C18" s="12" t="n">
@@ -7697,7 +8612,7 @@
       <x:c r="A19" s="11" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B19" s="28" t="n">
+      <x:c r="B19" s="29" t="n">
         <x:v>46419</x:v>
       </x:c>
       <x:c r="C19" s="12" t="n">
@@ -7723,7 +8638,7 @@
       <x:c r="A20" s="11" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B20" s="28" t="n">
+      <x:c r="B20" s="29" t="n">
         <x:v>46447</x:v>
       </x:c>
       <x:c r="C20" s="12" t="n">
@@ -7749,7 +8664,7 @@
       <x:c r="A21" s="11" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B21" s="28" t="n">
+      <x:c r="B21" s="29" t="n">
         <x:v>46478</x:v>
       </x:c>
       <x:c r="C21" s="12" t="n">
@@ -7775,7 +8690,7 @@
       <x:c r="A22" s="11" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B22" s="28" t="n">
+      <x:c r="B22" s="29" t="n">
         <x:v>46508</x:v>
       </x:c>
       <x:c r="C22" s="12" t="n">
@@ -7801,7 +8716,7 @@
       <x:c r="A23" s="11" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B23" s="28" t="n">
+      <x:c r="B23" s="29" t="n">
         <x:v>46539</x:v>
       </x:c>
       <x:c r="C23" s="12" t="n">
@@ -7827,7 +8742,7 @@
       <x:c r="A24" s="11" t="n">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B24" s="28" t="n">
+      <x:c r="B24" s="29" t="n">
         <x:v>46569</x:v>
       </x:c>
       <x:c r="C24" s="12" t="n">
@@ -7853,7 +8768,7 @@
       <x:c r="A25" s="11" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B25" s="28" t="n">
+      <x:c r="B25" s="29" t="n">
         <x:v>46600</x:v>
       </x:c>
       <x:c r="C25" s="12" t="n">
@@ -7879,7 +8794,7 @@
       <x:c r="A26" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B26" s="28" t="n">
+      <x:c r="B26" s="29" t="n">
         <x:v>46631</x:v>
       </x:c>
       <x:c r="C26" s="12" t="n">
@@ -7905,7 +8820,7 @@
       <x:c r="A27" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B27" s="28" t="n">
+      <x:c r="B27" s="29" t="n">
         <x:v>46661</x:v>
       </x:c>
       <x:c r="C27" s="12" t="n">
@@ -7931,7 +8846,7 @@
       <x:c r="A28" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B28" s="28" t="n">
+      <x:c r="B28" s="29" t="n">
         <x:v>46692</x:v>
       </x:c>
       <x:c r="C28" s="12" t="n">
@@ -7957,7 +8872,7 @@
       <x:c r="A29" s="11" t="n">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B29" s="28" t="n">
+      <x:c r="B29" s="29" t="n">
         <x:v>46722</x:v>
       </x:c>
       <x:c r="C29" s="12" t="n">
@@ -7983,7 +8898,7 @@
       <x:c r="A30" s="11" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B30" s="28" t="n">
+      <x:c r="B30" s="29" t="n">
         <x:v>46753</x:v>
       </x:c>
       <x:c r="C30" s="12" t="n">
@@ -8009,7 +8924,7 @@
       <x:c r="A31" s="11" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="B31" s="28" t="n">
+      <x:c r="B31" s="29" t="n">
         <x:v>46784</x:v>
       </x:c>
       <x:c r="C31" s="12" t="n">
@@ -8035,7 +8950,7 @@
       <x:c r="A32" s="11" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B32" s="28" t="n">
+      <x:c r="B32" s="29" t="n">
         <x:v>46813</x:v>
       </x:c>
       <x:c r="C32" s="12" t="n">
@@ -8061,7 +8976,7 @@
       <x:c r="A33" s="11" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B33" s="28" t="n">
+      <x:c r="B33" s="29" t="n">
         <x:v>46844</x:v>
       </x:c>
       <x:c r="C33" s="12" t="n">
@@ -8087,7 +9002,7 @@
       <x:c r="A34" s="11" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B34" s="28" t="n">
+      <x:c r="B34" s="29" t="n">
         <x:v>46874</x:v>
       </x:c>
       <x:c r="C34" s="12" t="n">
@@ -8113,7 +9028,7 @@
       <x:c r="A35" s="11" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B35" s="28" t="n">
+      <x:c r="B35" s="29" t="n">
         <x:v>46905</x:v>
       </x:c>
       <x:c r="C35" s="12" t="n">
@@ -8139,7 +9054,7 @@
       <x:c r="A36" s="11" t="n">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B36" s="28" t="n">
+      <x:c r="B36" s="29" t="n">
         <x:v>46935</x:v>
       </x:c>
       <x:c r="C36" s="12" t="n">
@@ -8165,7 +9080,7 @@
       <x:c r="A37" s="11" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B37" s="28" t="n">
+      <x:c r="B37" s="29" t="n">
         <x:v>46966</x:v>
       </x:c>
       <x:c r="C37" s="12" t="n">
@@ -8191,7 +9106,7 @@
       <x:c r="A38" s="11" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B38" s="28" t="n">
+      <x:c r="B38" s="29" t="n">
         <x:v>46997</x:v>
       </x:c>
       <x:c r="C38" s="12" t="n">
@@ -8217,7 +9132,7 @@
       <x:c r="A39" s="11" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="B39" s="28" t="n">
+      <x:c r="B39" s="29" t="n">
         <x:v>47027</x:v>
       </x:c>
       <x:c r="C39" s="12" t="n">
@@ -8243,7 +9158,7 @@
       <x:c r="A40" s="11" t="n">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="B40" s="28" t="n">
+      <x:c r="B40" s="29" t="n">
         <x:v>47058</x:v>
       </x:c>
       <x:c r="C40" s="12" t="n">
@@ -8269,7 +9184,7 @@
       <x:c r="A41" s="11" t="n">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="B41" s="28" t="n">
+      <x:c r="B41" s="29" t="n">
         <x:v>47088</x:v>
       </x:c>
       <x:c r="C41" s="12" t="n">
@@ -8295,7 +9210,7 @@
       <x:c r="A42" s="11" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B42" s="28" t="n">
+      <x:c r="B42" s="29" t="n">
         <x:v>47119</x:v>
       </x:c>
       <x:c r="C42" s="12" t="n">
@@ -8321,7 +9236,7 @@
       <x:c r="A43" s="11" t="n">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="B43" s="28" t="n">
+      <x:c r="B43" s="29" t="n">
         <x:v>47150</x:v>
       </x:c>
       <x:c r="C43" s="12" t="n">
@@ -8347,7 +9262,7 @@
       <x:c r="A44" s="11" t="n">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B44" s="28" t="n">
+      <x:c r="B44" s="29" t="n">
         <x:v>47178</x:v>
       </x:c>
       <x:c r="C44" s="12" t="n">
@@ -8373,7 +9288,7 @@
       <x:c r="A45" s="11" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="B45" s="28" t="n">
+      <x:c r="B45" s="29" t="n">
         <x:v>47209</x:v>
       </x:c>
       <x:c r="C45" s="12" t="n">
@@ -8399,7 +9314,7 @@
       <x:c r="A46" s="11" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="B46" s="28" t="n">
+      <x:c r="B46" s="29" t="n">
         <x:v>47239</x:v>
       </x:c>
       <x:c r="C46" s="12" t="n">
@@ -8425,7 +9340,7 @@
       <x:c r="A47" s="11" t="n">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B47" s="28" t="n">
+      <x:c r="B47" s="29" t="n">
         <x:v>47270</x:v>
       </x:c>
       <x:c r="C47" s="12" t="n">
@@ -8451,7 +9366,7 @@
       <x:c r="A48" s="11" t="n">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="B48" s="28" t="n">
+      <x:c r="B48" s="29" t="n">
         <x:v>47300</x:v>
       </x:c>
       <x:c r="C48" s="12" t="n">
@@ -8477,7 +9392,7 @@
       <x:c r="A49" s="11" t="n">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="B49" s="28" t="n">
+      <x:c r="B49" s="29" t="n">
         <x:v>47331</x:v>
       </x:c>
       <x:c r="C49" s="12" t="n">
@@ -8503,7 +9418,7 @@
       <x:c r="A50" s="11" t="n">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B50" s="28" t="n">
+      <x:c r="B50" s="29" t="n">
         <x:v>47362</x:v>
       </x:c>
       <x:c r="C50" s="12" t="n">
@@ -8529,7 +9444,7 @@
       <x:c r="A51" s="11" t="n">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="B51" s="28" t="n">
+      <x:c r="B51" s="29" t="n">
         <x:v>47392</x:v>
       </x:c>
       <x:c r="C51" s="12" t="n">
@@ -8555,7 +9470,7 @@
       <x:c r="A52" s="11" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B52" s="28" t="n">
+      <x:c r="B52" s="29" t="n">
         <x:v>47423</x:v>
       </x:c>
       <x:c r="C52" s="12" t="n">
@@ -8581,7 +9496,7 @@
       <x:c r="A53" s="11" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="B53" s="28" t="n">
+      <x:c r="B53" s="29" t="n">
         <x:v>47453</x:v>
       </x:c>
       <x:c r="C53" s="12" t="n">
@@ -8607,7 +9522,7 @@
       <x:c r="A54" s="11" t="n">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="B54" s="28" t="n">
+      <x:c r="B54" s="29" t="n">
         <x:v>47484</x:v>
       </x:c>
       <x:c r="C54" s="12" t="n">
@@ -8633,7 +9548,7 @@
       <x:c r="A55" s="11" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="B55" s="28" t="n">
+      <x:c r="B55" s="29" t="n">
         <x:v>47515</x:v>
       </x:c>
       <x:c r="C55" s="12" t="n">
@@ -8659,7 +9574,7 @@
       <x:c r="A56" s="11" t="n">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B56" s="28" t="n">
+      <x:c r="B56" s="29" t="n">
         <x:v>47543</x:v>
       </x:c>
       <x:c r="C56" s="12" t="n">
@@ -8685,7 +9600,7 @@
       <x:c r="A57" s="11" t="n">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="B57" s="28" t="n">
+      <x:c r="B57" s="29" t="n">
         <x:v>47574</x:v>
       </x:c>
       <x:c r="C57" s="12" t="n">
@@ -8711,7 +9626,7 @@
       <x:c r="A58" s="11" t="n">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="B58" s="28" t="n">
+      <x:c r="B58" s="29" t="n">
         <x:v>47604</x:v>
       </x:c>
       <x:c r="C58" s="12" t="n">
@@ -8737,7 +9652,7 @@
       <x:c r="A59" s="11" t="n">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="B59" s="28" t="n">
+      <x:c r="B59" s="29" t="n">
         <x:v>47635</x:v>
       </x:c>
       <x:c r="C59" s="12" t="n">
@@ -8763,7 +9678,7 @@
       <x:c r="A60" s="11" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="B60" s="28" t="n">
+      <x:c r="B60" s="29" t="n">
         <x:v>47665</x:v>
       </x:c>
       <x:c r="C60" s="12" t="n">
@@ -8789,7 +9704,7 @@
       <x:c r="A61" s="11" t="n">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="B61" s="28" t="n">
+      <x:c r="B61" s="29" t="n">
         <x:v>47696</x:v>
       </x:c>
       <x:c r="C61" s="12" t="n">
@@ -8815,7 +9730,7 @@
       <x:c r="A62" s="11" t="n">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="B62" s="28" t="n">
+      <x:c r="B62" s="29" t="n">
         <x:v>47727</x:v>
       </x:c>
       <x:c r="C62" s="12" t="n">
@@ -8841,7 +9756,7 @@
       <x:c r="A63" s="11" t="n">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="B63" s="28" t="n">
+      <x:c r="B63" s="29" t="n">
         <x:v>47757</x:v>
       </x:c>
       <x:c r="C63" s="12" t="n">
@@ -8867,7 +9782,7 @@
       <x:c r="A64" s="11" t="n">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="B64" s="28" t="n">
+      <x:c r="B64" s="29" t="n">
         <x:v>47788</x:v>
       </x:c>
       <x:c r="C64" s="12" t="n">
@@ -8893,7 +9808,7 @@
       <x:c r="A65" s="11" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="B65" s="28" t="n">
+      <x:c r="B65" s="29" t="n">
         <x:v>47818</x:v>
       </x:c>
       <x:c r="C65" s="12" t="n">
@@ -8916,46 +9831,46 @@
       </x:c>
     </x:row>
     <x:row r="66">
-      <x:c r="A66" s="44"/>
-      <x:c r="B66" s="44"/>
-      <x:c r="C66" s="44"/>
-      <x:c r="D66" s="44"/>
-      <x:c r="E66" s="44"/>
-      <x:c r="F66" s="44"/>
-      <x:c r="G66" s="44"/>
-      <x:c r="H66" s="44"/>
+      <x:c r="A66" s="45"/>
+      <x:c r="B66" s="45"/>
+      <x:c r="C66" s="45"/>
+      <x:c r="D66" s="45"/>
+      <x:c r="E66" s="45"/>
+      <x:c r="F66" s="45"/>
+      <x:c r="G66" s="45"/>
+      <x:c r="H66" s="45"/>
     </x:row>
     <x:row r="67">
-      <x:c r="A67" s="44"/>
-      <x:c r="B67" s="44"/>
-      <x:c r="C67" s="44"/>
-      <x:c r="D67" s="44"/>
-      <x:c r="E67" s="44"/>
-      <x:c r="F67" s="44"/>
-      <x:c r="G67" s="44"/>
-      <x:c r="H67" s="44"/>
+      <x:c r="A67" s="45"/>
+      <x:c r="B67" s="45"/>
+      <x:c r="C67" s="45"/>
+      <x:c r="D67" s="45"/>
+      <x:c r="E67" s="45"/>
+      <x:c r="F67" s="45"/>
+      <x:c r="G67" s="45"/>
+      <x:c r="H67" s="45"/>
     </x:row>
     <x:row r="68">
-      <x:c r="A68" s="36" t="str">
+      <x:c r="A68" s="37" t="str">
         <x:v>Fuente / dependencia</x:v>
       </x:c>
-      <x:c r="B68" s="36" t="str">
+      <x:c r="B68" s="37" t="str">
         <x:v>Uso</x:v>
       </x:c>
-      <x:c r="C68" s="36" t="str">
+      <x:c r="C68" s="37" t="str">
         <x:v>Tipo</x:v>
       </x:c>
-      <x:c r="D68" s="36" t="str">
+      <x:c r="D68" s="37" t="str">
         <x:v>URL o ruta</x:v>
       </x:c>
-      <x:c r="E68" s="36" t="str">
+      <x:c r="E68" s="37" t="str">
         <x:v>Fecha</x:v>
       </x:c>
-      <x:c r="F68" s="36" t="str">
+      <x:c r="F68" s="37" t="str">
         <x:v>Estado</x:v>
       </x:c>
-      <x:c r="G68" s="44"/>
-      <x:c r="H68" s="44"/>
+      <x:c r="G68" s="45"/>
+      <x:c r="H68" s="45"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="11" t="str">
@@ -8970,14 +9885,14 @@
       <x:c r="D69" s="11" t="str">
         <x:v>docs/fp-183/modelo-tco-linea-base-5-anos.xlsx</x:v>
       </x:c>
-      <x:c r="E69" s="28" t="n">
+      <x:c r="E69" s="29" t="n">
         <x:v>46281</x:v>
       </x:c>
       <x:c r="F69" s="11" t="str">
         <x:v>Verificado</x:v>
       </x:c>
-      <x:c r="G69" s="44"/>
-      <x:c r="H69" s="44"/>
+      <x:c r="G69" s="45"/>
+      <x:c r="H69" s="45"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="11" t="str">
@@ -8992,14 +9907,14 @@
       <x:c r="D70" s="11" t="str">
         <x:v>docs/fp-184/escenario-optimizado-fp-184.xlsx</x:v>
       </x:c>
-      <x:c r="E70" s="28" t="n">
+      <x:c r="E70" s="29" t="n">
         <x:v>46281</x:v>
       </x:c>
       <x:c r="F70" s="11" t="str">
         <x:v>Verificado</x:v>
       </x:c>
-      <x:c r="G70" s="44"/>
-      <x:c r="H70" s="44"/>
+      <x:c r="G70" s="45"/>
+      <x:c r="H70" s="45"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="11" t="str">
@@ -9014,14 +9929,14 @@
       <x:c r="D71" s="11" t="str">
         <x:v>FP-48 TINV02/Papers academicos - FP-48/markdown</x:v>
       </x:c>
-      <x:c r="E71" s="28" t="n">
+      <x:c r="E71" s="29" t="n">
         <x:v>46281</x:v>
       </x:c>
       <x:c r="F71" s="11" t="str">
         <x:v>Revisado</x:v>
       </x:c>
-      <x:c r="G71" s="44"/>
-      <x:c r="H71" s="44"/>
+      <x:c r="G71" s="45"/>
+      <x:c r="H71" s="45"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="11" t="str">
@@ -9036,14 +9951,14 @@
       <x:c r="D72" s="11" t="str">
         <x:v>https://learn.microsoft.com/en-us/azure/container-apps/billing</x:v>
       </x:c>
-      <x:c r="E72" s="28" t="n">
+      <x:c r="E72" s="29" t="n">
         <x:v>46281</x:v>
       </x:c>
       <x:c r="F72" s="11" t="str">
         <x:v>Consultado</x:v>
       </x:c>
-      <x:c r="G72" s="44"/>
-      <x:c r="H72" s="44"/>
+      <x:c r="G72" s="45"/>
+      <x:c r="H72" s="45"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="11" t="str">
@@ -9058,14 +9973,14 @@
       <x:c r="D73" s="11" t="str">
         <x:v>https://learn.microsoft.com/en-us/azure/postgresql/compute-storage/concepts-compute</x:v>
       </x:c>
-      <x:c r="E73" s="28" t="n">
+      <x:c r="E73" s="29" t="n">
         <x:v>46281</x:v>
       </x:c>
       <x:c r="F73" s="11" t="str">
         <x:v>Consultado</x:v>
       </x:c>
-      <x:c r="G73" s="44"/>
-      <x:c r="H73" s="44"/>
+      <x:c r="G73" s="45"/>
+      <x:c r="H73" s="45"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="11" t="str">
@@ -9080,14 +9995,14 @@
       <x:c r="D74" s="11" t="str">
         <x:v>https://azure.microsoft.com/en-us/pricing/details/bandwidth/</x:v>
       </x:c>
-      <x:c r="E74" s="28" t="n">
+      <x:c r="E74" s="29" t="n">
         <x:v>46281</x:v>
       </x:c>
       <x:c r="F74" s="11" t="str">
         <x:v>Consultado</x:v>
       </x:c>
-      <x:c r="G74" s="44"/>
-      <x:c r="H74" s="44"/>
+      <x:c r="G74" s="45"/>
+      <x:c r="H74" s="45"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="11" t="str">
@@ -9102,14 +10017,14 @@
       <x:c r="D75" s="11" t="str">
         <x:v>https://learn.microsoft.com/en-us/azure/azure-monitor/logs/workspace-design</x:v>
       </x:c>
-      <x:c r="E75" s="28" t="n">
+      <x:c r="E75" s="29" t="n">
         <x:v>46281</x:v>
       </x:c>
       <x:c r="F75" s="11" t="str">
         <x:v>Consultado</x:v>
       </x:c>
-      <x:c r="G75" s="44"/>
-      <x:c r="H75" s="44"/>
+      <x:c r="G75" s="45"/>
+      <x:c r="H75" s="45"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="11" t="str">
@@ -9124,14 +10039,14 @@
       <x:c r="D76" s="11" t="str">
         <x:v>https://sni.gob.cl/wp-content/uploads/Precios-Sociales-2026.pdf</x:v>
       </x:c>
-      <x:c r="E76" s="28" t="n">
+      <x:c r="E76" s="29" t="n">
         <x:v>46282</x:v>
       </x:c>
       <x:c r="F76" s="11" t="str">
         <x:v>Proxy público</x:v>
       </x:c>
-      <x:c r="G76" s="44"/>
-      <x:c r="H76" s="44"/>
+      <x:c r="G76" s="45"/>
+      <x:c r="H76" s="45"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="11" t="str">
@@ -9146,14 +10061,14 @@
       <x:c r="D77" s="11" t="str">
         <x:v>https://www.ine.gob.cl/docs/default-source/encuesta-suplementaria-de-ingresos/publicaciones-y-anuarios/s%C3%ADntesis-de-resultados/2024/esi2024.pdf</x:v>
       </x:c>
-      <x:c r="E77" s="28" t="n">
+      <x:c r="E77" s="29" t="n">
         <x:v>46282</x:v>
       </x:c>
       <x:c r="F77" s="11" t="str">
         <x:v>Proxy público</x:v>
       </x:c>
-      <x:c r="G77" s="44"/>
-      <x:c r="H77" s="44"/>
+      <x:c r="G77" s="45"/>
+      <x:c r="H77" s="45"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="11" t="str">
@@ -9168,14 +10083,14 @@
       <x:c r="D78" s="11" t="str">
         <x:v>https://www.dt.gob.cl/portal/1626/w3-propertyname-2556.html</x:v>
       </x:c>
-      <x:c r="E78" s="28" t="n">
+      <x:c r="E78" s="29" t="n">
         <x:v>46282</x:v>
       </x:c>
       <x:c r="F78" s="11" t="str">
         <x:v>Verificado</x:v>
       </x:c>
-      <x:c r="G78" s="44"/>
-      <x:c r="H78" s="44"/>
+      <x:c r="G78" s="45"/>
+      <x:c r="H78" s="45"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="11" t="str">
@@ -9190,14 +10105,14 @@
       <x:c r="D79" s="11" t="str">
         <x:v>https://si3.bcentral.cl/siete/ES/Siete/Cuadro/CAP_TIPO_CAMBIO/MN_TIPO_CAMBIO4/DOLAR_OBS_ADO?idSerie=F073.TCO.PRE.Z.D</x:v>
       </x:c>
-      <x:c r="E79" s="28" t="n">
+      <x:c r="E79" s="29" t="n">
         <x:v>46282</x:v>
       </x:c>
       <x:c r="F79" s="11" t="str">
         <x:v>Verificado</x:v>
       </x:c>
-      <x:c r="G79" s="44"/>
-      <x:c r="H79" s="44"/>
+      <x:c r="G79" s="45"/>
+      <x:c r="H79" s="45"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="11" t="str">
@@ -9212,14 +10127,14 @@
       <x:c r="D80" s="11" t="str">
         <x:v>https://www.finops.org/framework/capabilities/usage-optimization/</x:v>
       </x:c>
-      <x:c r="E80" s="28" t="n">
+      <x:c r="E80" s="29" t="n">
         <x:v>46282</x:v>
       </x:c>
       <x:c r="F80" s="11" t="str">
         <x:v>Método</x:v>
       </x:c>
-      <x:c r="G80" s="44"/>
-      <x:c r="H80" s="44"/>
+      <x:c r="G80" s="45"/>
+      <x:c r="H80" s="45"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="11" t="str">
@@ -9234,14 +10149,14 @@
       <x:c r="D81" s="11" t="str">
         <x:v>https://www.finops.org/framework/capabilities/planning-estimating/</x:v>
       </x:c>
-      <x:c r="E81" s="28" t="n">
+      <x:c r="E81" s="29" t="n">
         <x:v>46282</x:v>
       </x:c>
       <x:c r="F81" s="11" t="str">
         <x:v>Método</x:v>
       </x:c>
-      <x:c r="G81" s="44"/>
-      <x:c r="H81" s="44"/>
+      <x:c r="G81" s="45"/>
+      <x:c r="H81" s="45"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -9264,35 +10179,35 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="43" t="str">
+      <x:c r="A1" s="44" t="str">
         <x:v>FP-187 — Auditoría y conciliación</x:v>
       </x:c>
-      <x:c r="B1" s="43"/>
-      <x:c r="C1" s="43"/>
-      <x:c r="D1" s="43"/>
-      <x:c r="E1" s="43"/>
+      <x:c r="B1" s="44"/>
+      <x:c r="C1" s="44"/>
+      <x:c r="D1" s="44"/>
+      <x:c r="E1" s="44"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="44"/>
-      <x:c r="B2" s="44"/>
-      <x:c r="C2" s="44"/>
-      <x:c r="D2" s="44"/>
-      <x:c r="E2" s="44"/>
+      <x:c r="A2" s="45"/>
+      <x:c r="B2" s="45"/>
+      <x:c r="C2" s="45"/>
+      <x:c r="D2" s="45"/>
+      <x:c r="E2" s="45"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="36" t="str">
+      <x:c r="A3" s="37" t="str">
         <x:v>Control</x:v>
       </x:c>
-      <x:c r="B3" s="36" t="str">
+      <x:c r="B3" s="37" t="str">
         <x:v>Esperado</x:v>
       </x:c>
-      <x:c r="C3" s="36" t="str">
+      <x:c r="C3" s="37" t="str">
         <x:v>Calculado</x:v>
       </x:c>
-      <x:c r="D3" s="36" t="str">
+      <x:c r="D3" s="37" t="str">
         <x:v>Diferencia</x:v>
       </x:c>
-      <x:c r="E3" s="36" t="str">
+      <x:c r="E3" s="37" t="str">
         <x:v>Estado</x:v>
       </x:c>
     </x:row>
@@ -9380,14 +10295,14 @@
       <x:c r="A8" s="11" t="str">
         <x:v>Horizonte meses</x:v>
       </x:c>
-      <x:c r="B8" s="29" t="n">
+      <x:c r="B8" s="30" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="C8" s="29" t="n">
+      <x:c r="C8" s="30" t="n">
         <x:f>Supuestos!B7</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="D8" s="29" t="n">
+      <x:c r="D8" s="30" t="n">
         <x:f>C8-B8</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -9408,7 +10323,7 @@
         <x:v>Sí: proxies públicos</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str"/>
-      <x:c r="E9" s="14" t="str">
+      <x:c r="E9" s="15" t="str">
         <x:f>IF(C9="Sí: proxies públicos","PROVISIONAL","PENDIENTE")</x:f>
         <x:v>PROVISIONAL</x:v>
       </x:c>
@@ -9458,14 +10373,14 @@
       <x:c r="A12" s="11" t="str">
         <x:v>Horas implementación</x:v>
       </x:c>
-      <x:c r="B12" s="27" t="n">
+      <x:c r="B12" s="28" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="C12" s="27" t="n">
+      <x:c r="C12" s="28" t="n">
         <x:f>Supuestos!B29</x:f>
         <x:v>50</x:v>
       </x:c>
-      <x:c r="D12" s="27" t="n">
+      <x:c r="D12" s="28" t="n">
         <x:f>C12-B12</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -9478,14 +10393,14 @@
       <x:c r="A13" s="11" t="str">
         <x:v>Horas operación mensual</x:v>
       </x:c>
-      <x:c r="B13" s="27" t="n">
+      <x:c r="B13" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C13" s="27" t="n">
+      <x:c r="C13" s="28" t="n">
         <x:f>Supuestos!B30</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D13" s="27" t="n">
+      <x:c r="D13" s="28" t="n">
         <x:f>C13-B13</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -9495,25 +10410,62 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="44"/>
-      <x:c r="B14" s="44"/>
-      <x:c r="C14" s="44"/>
-      <x:c r="D14" s="44"/>
-      <x:c r="E14" s="44"/>
+      <x:c r="A14" s="11" t="str">
+        <x:v>PRI descontado Chile</x:v>
+      </x:c>
+      <x:c r="B14" s="14" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C14" s="14" t="n">
+        <x:f>'Resumen'!K5</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D14" s="14" t="n">
+        <x:f>IF(ISNUMBER(C14),C14-B14,"")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="str">
+        <x:f>IF(C14=B14,"OK","REVISAR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="37" t="str">
-        <x:v>Interpretación: los controles verifican coherencia matemática y trazabilidad. PROVISIONAL significa que se usaron proxies públicos, no que exista aprobación financiera interna.</x:v>
-      </x:c>
-      <x:c r="B15" s="37"/>
-      <x:c r="C15" s="37"/>
-      <x:c r="D15" s="37"/>
-      <x:c r="E15" s="37"/>
+      <x:c r="A15" s="11" t="str">
+        <x:v>PRI descontado East US</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="str">
+        <x:v>No recupera en 60 meses</x:v>
+      </x:c>
+      <x:c r="C15" s="11" t="str">
+        <x:f>'Resumen'!K6</x:f>
+        <x:v>No recupera en 60 meses</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="str"/>
+      <x:c r="E15" s="11" t="str">
+        <x:f>IF(C15=B15,"OK","REVISAR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="45"/>
+      <x:c r="B16" s="45"/>
+      <x:c r="C16" s="45"/>
+      <x:c r="D16" s="45"/>
+      <x:c r="E16" s="45"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="38" t="str">
+        <x:v>Interpretación: los controles verifican coherencia matemática y trazabilidad. PROVISIONAL significa que se usaron proxies públicos, no que exista aprobación financiera interna. El PRI se obtiene del primer cruce no negativo del flujo descontado acumulado.</x:v>
+      </x:c>
+      <x:c r="B17" s="38"/>
+      <x:c r="C17" s="38"/>
+      <x:c r="D17" s="38"/>
+      <x:c r="E17" s="38"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
-    <x:mergeCell ref="A15:E15"/>
+    <x:mergeCell ref="A17:E17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>